<commit_message>
Fixed: Test sheet to have male/female instead of boy/girl
</commit_message>
<xml_diff>
--- a/tests/students_test_data.xlsx
+++ b/tests/students_test_data.xlsx
@@ -457,7 +457,7 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>894715</v>
+        <v>556618</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
@@ -466,19 +466,19 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Girl</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Msc</t>
+          <t>Isl</t>
         </is>
       </c>
       <c r="E2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>470135</v>
+        <v>439626</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -487,7 +487,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Boy</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -499,7 +499,7 @@
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>510037</v>
+        <v>422078</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -508,19 +508,19 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Girl</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Isl</t>
+          <t>Msc</t>
         </is>
       </c>
       <c r="E4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>215425</v>
+        <v>231426</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
@@ -529,19 +529,23 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Boy</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Isl</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr"/>
+          <t>Msc</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Naughty</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>879373</v>
+        <v>768989</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
@@ -550,19 +554,19 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Boy</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Isl</t>
+          <t>Msc</t>
         </is>
       </c>
       <c r="E6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>391925</v>
+        <v>354126</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
@@ -571,7 +575,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Girl</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -583,7 +587,7 @@
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>913907</v>
+        <v>595140</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
@@ -592,7 +596,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Boy</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -604,7 +608,7 @@
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>646517</v>
+        <v>438894</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
@@ -613,7 +617,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Boy</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -621,15 +625,11 @@
           <t>Msc</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>Weak in studies</t>
-        </is>
-      </c>
+      <c r="E9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>638801</v>
+        <v>418319</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
@@ -638,19 +638,19 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Boy</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Msc</t>
+          <t>Isl</t>
         </is>
       </c>
       <c r="E10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>964939</v>
+        <v>442768</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
@@ -659,7 +659,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Girl</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -671,7 +671,7 @@
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>368775</v>
+        <v>700245</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
@@ -680,19 +680,19 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Girl</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Isl</t>
+          <t>Msc</t>
         </is>
       </c>
       <c r="E12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>297696</v>
+        <v>932445</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
@@ -701,19 +701,19 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Boy</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Isl</t>
+          <t>Msc</t>
         </is>
       </c>
       <c r="E13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>487863</v>
+        <v>550953</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
@@ -722,7 +722,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Girl</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -734,7 +734,7 @@
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>732707</v>
+        <v>703118</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
@@ -743,7 +743,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Boy</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -755,7 +755,7 @@
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>844011</v>
+        <v>611011</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
@@ -764,7 +764,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Girl</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -776,7 +776,7 @@
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>461302</v>
+        <v>417040</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
@@ -785,19 +785,19 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Boy</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Msc</t>
+          <t>Isl</t>
         </is>
       </c>
       <c r="E17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>193817</v>
+        <v>955101</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
@@ -806,7 +806,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Girl</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -814,11 +814,15 @@
           <t>Msc</t>
         </is>
       </c>
-      <c r="E18" t="inlineStr"/>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Naughty</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>739253</v>
+        <v>264831</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
@@ -827,7 +831,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Boy</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -839,7 +843,7 @@
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>889659</v>
+        <v>110494</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
@@ -848,19 +852,23 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Boy</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Isl</t>
-        </is>
-      </c>
-      <c r="E20" t="inlineStr"/>
+          <t>Msc</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Naughty</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>890239</v>
+        <v>756117</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
@@ -869,7 +877,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Girl</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -881,7 +889,7 @@
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>830269</v>
+        <v>368243</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
@@ -890,19 +898,19 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Boy</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Msc</t>
+          <t>Isl</t>
         </is>
       </c>
       <c r="E22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>532239</v>
+        <v>886449</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
@@ -911,19 +919,19 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Boy</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Msc</t>
+          <t>Isl</t>
         </is>
       </c>
       <c r="E23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>206051</v>
+        <v>811978</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
@@ -932,19 +940,19 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Girl</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Isl</t>
+          <t>Msc</t>
         </is>
       </c>
       <c r="E24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>471842</v>
+        <v>719615</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
@@ -953,7 +961,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Girl</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -961,15 +969,11 @@
           <t>Msc</t>
         </is>
       </c>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t>Naughty</t>
-        </is>
-      </c>
+      <c r="E25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="n">
-        <v>692513</v>
+        <v>726064</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
@@ -978,7 +982,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Boy</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -986,11 +990,15 @@
           <t>Msc</t>
         </is>
       </c>
-      <c r="E26" t="inlineStr"/>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Weak in studies</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
-        <v>143175</v>
+        <v>770663</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
@@ -999,19 +1007,19 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Girl</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Isl</t>
+          <t>Msc</t>
         </is>
       </c>
       <c r="E27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="n">
-        <v>821268</v>
+        <v>632975</v>
       </c>
       <c r="B28" t="inlineStr">
         <is>
@@ -1020,7 +1028,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Girl</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -1028,15 +1036,11 @@
           <t>Msc</t>
         </is>
       </c>
-      <c r="E28" t="inlineStr">
-        <is>
-          <t>Naughty</t>
-        </is>
-      </c>
+      <c r="E28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="n">
-        <v>330638</v>
+        <v>449232</v>
       </c>
       <c r="B29" t="inlineStr">
         <is>
@@ -1045,19 +1049,19 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Girl</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Msc</t>
+          <t>Isl</t>
         </is>
       </c>
       <c r="E29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="n">
-        <v>928408</v>
+        <v>284090</v>
       </c>
       <c r="B30" t="inlineStr">
         <is>
@@ -1066,7 +1070,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Girl</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -1078,7 +1082,7 @@
     </row>
     <row r="31">
       <c r="A31" t="n">
-        <v>448313</v>
+        <v>981074</v>
       </c>
       <c r="B31" t="inlineStr">
         <is>
@@ -1087,7 +1091,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Girl</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -1099,7 +1103,7 @@
     </row>
     <row r="32">
       <c r="A32" t="n">
-        <v>475650</v>
+        <v>400264</v>
       </c>
       <c r="B32" t="inlineStr">
         <is>
@@ -1108,19 +1112,19 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Girl</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Msc</t>
+          <t>Isl</t>
         </is>
       </c>
       <c r="E32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="n">
-        <v>124917</v>
+        <v>715586</v>
       </c>
       <c r="B33" t="inlineStr">
         <is>
@@ -1129,7 +1133,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Girl</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -1141,7 +1145,7 @@
     </row>
     <row r="34">
       <c r="A34" t="n">
-        <v>897332</v>
+        <v>804889</v>
       </c>
       <c r="B34" t="inlineStr">
         <is>
@@ -1150,7 +1154,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Boy</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -1162,7 +1166,7 @@
     </row>
     <row r="35">
       <c r="A35" t="n">
-        <v>317794</v>
+        <v>273518</v>
       </c>
       <c r="B35" t="inlineStr">
         <is>
@@ -1171,19 +1175,19 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Girl</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Msc</t>
+          <t>Isl</t>
         </is>
       </c>
       <c r="E35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="n">
-        <v>709075</v>
+        <v>127017</v>
       </c>
       <c r="B36" t="inlineStr">
         <is>
@@ -1192,19 +1196,19 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Boy</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Isl</t>
+          <t>Msc</t>
         </is>
       </c>
       <c r="E36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="n">
-        <v>648699</v>
+        <v>714244</v>
       </c>
       <c r="B37" t="inlineStr">
         <is>
@@ -1213,7 +1217,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Boy</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -1221,11 +1225,15 @@
           <t>Isl</t>
         </is>
       </c>
-      <c r="E37" t="inlineStr"/>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>Naughty</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="n">
-        <v>321312</v>
+        <v>710275</v>
       </c>
       <c r="B38" t="inlineStr">
         <is>
@@ -1234,23 +1242,19 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Girl</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Msc</t>
-        </is>
-      </c>
-      <c r="E38" t="inlineStr">
-        <is>
-          <t>Weak in studies</t>
-        </is>
-      </c>
+          <t>Isl</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="n">
-        <v>341153</v>
+        <v>557873</v>
       </c>
       <c r="B39" t="inlineStr">
         <is>
@@ -1259,7 +1263,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Girl</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -1271,7 +1275,7 @@
     </row>
     <row r="40">
       <c r="A40" t="n">
-        <v>817416</v>
+        <v>325311</v>
       </c>
       <c r="B40" t="inlineStr">
         <is>
@@ -1280,7 +1284,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Boy</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -1292,7 +1296,7 @@
     </row>
     <row r="41">
       <c r="A41" t="n">
-        <v>257440</v>
+        <v>884755</v>
       </c>
       <c r="B41" t="inlineStr">
         <is>
@@ -1301,7 +1305,7 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Girl</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -1313,7 +1317,7 @@
     </row>
     <row r="42">
       <c r="A42" t="n">
-        <v>628851</v>
+        <v>808404</v>
       </c>
       <c r="B42" t="inlineStr">
         <is>
@@ -1322,7 +1326,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Boy</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -1334,7 +1338,7 @@
     </row>
     <row r="43">
       <c r="A43" t="n">
-        <v>822479</v>
+        <v>581753</v>
       </c>
       <c r="B43" t="inlineStr">
         <is>
@@ -1343,7 +1347,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Boy</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -1355,7 +1359,7 @@
     </row>
     <row r="44">
       <c r="A44" t="n">
-        <v>262610</v>
+        <v>592647</v>
       </c>
       <c r="B44" t="inlineStr">
         <is>
@@ -1364,7 +1368,7 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Boy</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -1376,7 +1380,7 @@
     </row>
     <row r="45">
       <c r="A45" t="n">
-        <v>565970</v>
+        <v>762029</v>
       </c>
       <c r="B45" t="inlineStr">
         <is>
@@ -1385,19 +1389,19 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Girl</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Isl</t>
+          <t>Msc</t>
         </is>
       </c>
       <c r="E45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="n">
-        <v>747438</v>
+        <v>585750</v>
       </c>
       <c r="B46" t="inlineStr">
         <is>
@@ -1406,19 +1410,19 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Boy</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Msc</t>
+          <t>Isl</t>
         </is>
       </c>
       <c r="E46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="n">
-        <v>782332</v>
+        <v>787167</v>
       </c>
       <c r="B47" t="inlineStr">
         <is>
@@ -1427,7 +1431,7 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Girl</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
@@ -1439,7 +1443,7 @@
     </row>
     <row r="48">
       <c r="A48" t="n">
-        <v>630431</v>
+        <v>753554</v>
       </c>
       <c r="B48" t="inlineStr">
         <is>
@@ -1448,19 +1452,19 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Boy</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Isl</t>
+          <t>Msc</t>
         </is>
       </c>
       <c r="E48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="n">
-        <v>809928</v>
+        <v>846376</v>
       </c>
       <c r="B49" t="inlineStr">
         <is>
@@ -1469,7 +1473,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Girl</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
@@ -1481,7 +1485,7 @@
     </row>
     <row r="50">
       <c r="A50" t="n">
-        <v>241063</v>
+        <v>881175</v>
       </c>
       <c r="B50" t="inlineStr">
         <is>
@@ -1490,19 +1494,19 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Girl</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Msc</t>
+          <t>Isl</t>
         </is>
       </c>
       <c r="E50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="n">
-        <v>941287</v>
+        <v>135481</v>
       </c>
       <c r="B51" t="inlineStr">
         <is>
@@ -1511,19 +1515,19 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Girl</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Isl</t>
+          <t>Msc</t>
         </is>
       </c>
       <c r="E51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="n">
-        <v>555775</v>
+        <v>431046</v>
       </c>
       <c r="B52" t="inlineStr">
         <is>
@@ -1532,7 +1536,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Boy</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
@@ -1544,7 +1548,7 @@
     </row>
     <row r="53">
       <c r="A53" t="n">
-        <v>835200</v>
+        <v>600855</v>
       </c>
       <c r="B53" t="inlineStr">
         <is>
@@ -1553,7 +1557,7 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Girl</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
@@ -1561,11 +1565,15 @@
           <t>Msc</t>
         </is>
       </c>
-      <c r="E53" t="inlineStr"/>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>Naughty</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="n">
-        <v>164588</v>
+        <v>266048</v>
       </c>
       <c r="B54" t="inlineStr">
         <is>
@@ -1574,23 +1582,19 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Girl</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Msc</t>
-        </is>
-      </c>
-      <c r="E54" t="inlineStr">
-        <is>
-          <t>Naughty</t>
-        </is>
-      </c>
+          <t>Isl</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="n">
-        <v>474553</v>
+        <v>398424</v>
       </c>
       <c r="B55" t="inlineStr">
         <is>
@@ -1599,7 +1603,7 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Girl</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
@@ -1611,7 +1615,7 @@
     </row>
     <row r="56">
       <c r="A56" t="n">
-        <v>623543</v>
+        <v>844393</v>
       </c>
       <c r="B56" t="inlineStr">
         <is>
@@ -1620,19 +1624,23 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Boy</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Msc</t>
-        </is>
-      </c>
-      <c r="E56" t="inlineStr"/>
+          <t>Isl</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>Naughty</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="n">
-        <v>958808</v>
+        <v>254552</v>
       </c>
       <c r="B57" t="inlineStr">
         <is>
@@ -1641,19 +1649,23 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Girl</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Msc</t>
-        </is>
-      </c>
-      <c r="E57" t="inlineStr"/>
+          <t>Isl</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>Naughty</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="n">
-        <v>840824</v>
+        <v>829601</v>
       </c>
       <c r="B58" t="inlineStr">
         <is>
@@ -1662,7 +1674,7 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Girl</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
@@ -1674,7 +1686,7 @@
     </row>
     <row r="59">
       <c r="A59" t="n">
-        <v>164689</v>
+        <v>393039</v>
       </c>
       <c r="B59" t="inlineStr">
         <is>
@@ -1683,19 +1695,19 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Boy</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Isl</t>
+          <t>Msc</t>
         </is>
       </c>
       <c r="E59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="n">
-        <v>491864</v>
+        <v>822193</v>
       </c>
       <c r="B60" t="inlineStr">
         <is>
@@ -1704,19 +1716,19 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Boy</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Isl</t>
+          <t>Msc</t>
         </is>
       </c>
       <c r="E60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="n">
-        <v>224630</v>
+        <v>303037</v>
       </c>
       <c r="B61" t="inlineStr">
         <is>
@@ -1725,19 +1737,19 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Boy</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Isl</t>
+          <t>Msc</t>
         </is>
       </c>
       <c r="E61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="n">
-        <v>248089</v>
+        <v>101919</v>
       </c>
       <c r="B62" t="inlineStr">
         <is>
@@ -1746,7 +1758,7 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Girl</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
@@ -1758,7 +1770,7 @@
     </row>
     <row r="63">
       <c r="A63" t="n">
-        <v>145991</v>
+        <v>848723</v>
       </c>
       <c r="B63" t="inlineStr">
         <is>
@@ -1767,7 +1779,7 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Girl</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
@@ -1779,7 +1791,7 @@
     </row>
     <row r="64">
       <c r="A64" t="n">
-        <v>600642</v>
+        <v>858106</v>
       </c>
       <c r="B64" t="inlineStr">
         <is>
@@ -1788,7 +1800,7 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Girl</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
@@ -1800,7 +1812,7 @@
     </row>
     <row r="65">
       <c r="A65" t="n">
-        <v>991009</v>
+        <v>261958</v>
       </c>
       <c r="B65" t="inlineStr">
         <is>
@@ -1809,19 +1821,19 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Boy</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Msc</t>
+          <t>Isl</t>
         </is>
       </c>
       <c r="E65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="n">
-        <v>241148</v>
+        <v>650696</v>
       </c>
       <c r="B66" t="inlineStr">
         <is>
@@ -1830,19 +1842,19 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Girl</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>Msc</t>
+          <t>Isl</t>
         </is>
       </c>
       <c r="E66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="n">
-        <v>263743</v>
+        <v>457202</v>
       </c>
       <c r="B67" t="inlineStr">
         <is>
@@ -1851,19 +1863,19 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Girl</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Msc</t>
+          <t>Isl</t>
         </is>
       </c>
       <c r="E67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="n">
-        <v>403839</v>
+        <v>942057</v>
       </c>
       <c r="B68" t="inlineStr">
         <is>
@@ -1872,7 +1884,7 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Boy</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
@@ -1884,7 +1896,7 @@
     </row>
     <row r="69">
       <c r="A69" t="n">
-        <v>534261</v>
+        <v>422836</v>
       </c>
       <c r="B69" t="inlineStr">
         <is>
@@ -1893,19 +1905,19 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Girl</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Msc</t>
+          <t>Isl</t>
         </is>
       </c>
       <c r="E69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="n">
-        <v>786868</v>
+        <v>411384</v>
       </c>
       <c r="B70" t="inlineStr">
         <is>
@@ -1914,7 +1926,7 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Girl</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
@@ -1926,7 +1938,7 @@
     </row>
     <row r="71">
       <c r="A71" t="n">
-        <v>811758</v>
+        <v>266809</v>
       </c>
       <c r="B71" t="inlineStr">
         <is>
@@ -1935,7 +1947,7 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Boy</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
@@ -1947,7 +1959,7 @@
     </row>
     <row r="72">
       <c r="A72" t="n">
-        <v>459544</v>
+        <v>917729</v>
       </c>
       <c r="B72" t="inlineStr">
         <is>
@@ -1956,19 +1968,19 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Boy</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>Msc</t>
+          <t>Isl</t>
         </is>
       </c>
       <c r="E72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="n">
-        <v>385085</v>
+        <v>544498</v>
       </c>
       <c r="B73" t="inlineStr">
         <is>
@@ -1977,19 +1989,19 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>Boy</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>Msc</t>
+          <t>Isl</t>
         </is>
       </c>
       <c r="E73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" t="n">
-        <v>944489</v>
+        <v>156946</v>
       </c>
       <c r="B74" t="inlineStr">
         <is>
@@ -1998,7 +2010,7 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>Boy</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
@@ -2010,7 +2022,7 @@
     </row>
     <row r="75">
       <c r="A75" t="n">
-        <v>423861</v>
+        <v>748911</v>
       </c>
       <c r="B75" t="inlineStr">
         <is>
@@ -2019,7 +2031,7 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>Girl</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
@@ -2031,7 +2043,7 @@
     </row>
     <row r="76">
       <c r="A76" t="n">
-        <v>275009</v>
+        <v>652667</v>
       </c>
       <c r="B76" t="inlineStr">
         <is>
@@ -2040,7 +2052,7 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Girl</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
@@ -2052,7 +2064,7 @@
     </row>
     <row r="77">
       <c r="A77" t="n">
-        <v>535778</v>
+        <v>889382</v>
       </c>
       <c r="B77" t="inlineStr">
         <is>
@@ -2061,7 +2073,7 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Boy</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
@@ -2073,7 +2085,7 @@
     </row>
     <row r="78">
       <c r="A78" t="n">
-        <v>404303</v>
+        <v>994332</v>
       </c>
       <c r="B78" t="inlineStr">
         <is>
@@ -2082,7 +2094,7 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>Girl</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
@@ -2090,15 +2102,11 @@
           <t>Msc</t>
         </is>
       </c>
-      <c r="E78" t="inlineStr">
-        <is>
-          <t>Naughty</t>
-        </is>
-      </c>
+      <c r="E78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" t="n">
-        <v>618022</v>
+        <v>519893</v>
       </c>
       <c r="B79" t="inlineStr">
         <is>
@@ -2107,7 +2115,7 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>Girl</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
@@ -2119,7 +2127,7 @@
     </row>
     <row r="80">
       <c r="A80" t="n">
-        <v>871278</v>
+        <v>105647</v>
       </c>
       <c r="B80" t="inlineStr">
         <is>
@@ -2128,19 +2136,19 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>Boy</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>Isl</t>
+          <t>Msc</t>
         </is>
       </c>
       <c r="E80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" t="n">
-        <v>616942</v>
+        <v>877190</v>
       </c>
       <c r="B81" t="inlineStr">
         <is>
@@ -2149,7 +2157,7 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Boy</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
@@ -2161,7 +2169,7 @@
     </row>
     <row r="82">
       <c r="A82" t="n">
-        <v>743417</v>
+        <v>700858</v>
       </c>
       <c r="B82" t="inlineStr">
         <is>
@@ -2170,19 +2178,19 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>Boy</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>Isl</t>
+          <t>Msc</t>
         </is>
       </c>
       <c r="E82" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" t="n">
-        <v>174197</v>
+        <v>491524</v>
       </c>
       <c r="B83" t="inlineStr">
         <is>
@@ -2191,19 +2199,19 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Girl</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>Isl</t>
+          <t>Msc</t>
         </is>
       </c>
       <c r="E83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" t="n">
-        <v>779724</v>
+        <v>313081</v>
       </c>
       <c r="B84" t="inlineStr">
         <is>
@@ -2212,23 +2220,19 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>Boy</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>Msc</t>
-        </is>
-      </c>
-      <c r="E84" t="inlineStr">
-        <is>
-          <t>Naughty</t>
-        </is>
-      </c>
+          <t>Isl</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" t="n">
-        <v>605394</v>
+        <v>713280</v>
       </c>
       <c r="B85" t="inlineStr">
         <is>
@@ -2237,7 +2241,7 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>Boy</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
@@ -2249,7 +2253,7 @@
     </row>
     <row r="86">
       <c r="A86" t="n">
-        <v>637179</v>
+        <v>522822</v>
       </c>
       <c r="B86" t="inlineStr">
         <is>
@@ -2258,7 +2262,7 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>Boy</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
@@ -2266,11 +2270,15 @@
           <t>Msc</t>
         </is>
       </c>
-      <c r="E86" t="inlineStr"/>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>Naughty</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="n">
-        <v>762881</v>
+        <v>451111</v>
       </c>
       <c r="B87" t="inlineStr">
         <is>
@@ -2279,7 +2287,7 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>Girl</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
@@ -2291,7 +2299,7 @@
     </row>
     <row r="88">
       <c r="A88" t="n">
-        <v>303103</v>
+        <v>276364</v>
       </c>
       <c r="B88" t="inlineStr">
         <is>
@@ -2300,7 +2308,7 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>Boy</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
@@ -2308,15 +2316,11 @@
           <t>Msc</t>
         </is>
       </c>
-      <c r="E88" t="inlineStr">
-        <is>
-          <t>Weak in studies</t>
-        </is>
-      </c>
+      <c r="E88" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" t="n">
-        <v>494660</v>
+        <v>499376</v>
       </c>
       <c r="B89" t="inlineStr">
         <is>
@@ -2325,19 +2329,19 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>Girl</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>Isl</t>
+          <t>Msc</t>
         </is>
       </c>
       <c r="E89" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" t="n">
-        <v>567195</v>
+        <v>429189</v>
       </c>
       <c r="B90" t="inlineStr">
         <is>
@@ -2346,7 +2350,7 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>Boy</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
@@ -2358,7 +2362,7 @@
     </row>
     <row r="91">
       <c r="A91" t="n">
-        <v>117646</v>
+        <v>221871</v>
       </c>
       <c r="B91" t="inlineStr">
         <is>
@@ -2367,7 +2371,7 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>Girl</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
@@ -2379,7 +2383,7 @@
     </row>
     <row r="92">
       <c r="A92" t="n">
-        <v>566024</v>
+        <v>932342</v>
       </c>
       <c r="B92" t="inlineStr">
         <is>
@@ -2388,7 +2392,7 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>Boy</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
@@ -2400,7 +2404,7 @@
     </row>
     <row r="93">
       <c r="A93" t="n">
-        <v>308674</v>
+        <v>747095</v>
       </c>
       <c r="B93" t="inlineStr">
         <is>
@@ -2409,7 +2413,7 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>Girl</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
@@ -2421,7 +2425,7 @@
     </row>
     <row r="94">
       <c r="A94" t="n">
-        <v>338901</v>
+        <v>673359</v>
       </c>
       <c r="B94" t="inlineStr">
         <is>
@@ -2430,7 +2434,7 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>Girl</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
@@ -2438,11 +2442,15 @@
           <t>Isl</t>
         </is>
       </c>
-      <c r="E94" t="inlineStr"/>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>Weak in studies</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="n">
-        <v>508721</v>
+        <v>671800</v>
       </c>
       <c r="B95" t="inlineStr">
         <is>
@@ -2451,19 +2459,19 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>Boy</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>Isl</t>
+          <t>Msc</t>
         </is>
       </c>
       <c r="E95" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" t="n">
-        <v>771847</v>
+        <v>105327</v>
       </c>
       <c r="B96" t="inlineStr">
         <is>
@@ -2472,23 +2480,19 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>Boy</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>Msc</t>
-        </is>
-      </c>
-      <c r="E96" t="inlineStr">
-        <is>
-          <t>Weak in studies</t>
-        </is>
-      </c>
+          <t>Isl</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" t="n">
-        <v>261242</v>
+        <v>146561</v>
       </c>
       <c r="B97" t="inlineStr">
         <is>
@@ -2497,7 +2501,7 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>Boy</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
@@ -2509,7 +2513,7 @@
     </row>
     <row r="98">
       <c r="A98" t="n">
-        <v>388594</v>
+        <v>210728</v>
       </c>
       <c r="B98" t="inlineStr">
         <is>
@@ -2518,19 +2522,19 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>Boy</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>Isl</t>
+          <t>Msc</t>
         </is>
       </c>
       <c r="E98" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" t="n">
-        <v>346297</v>
+        <v>405592</v>
       </c>
       <c r="B99" t="inlineStr">
         <is>
@@ -2539,23 +2543,19 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>Boy</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>Msc</t>
-        </is>
-      </c>
-      <c r="E99" t="inlineStr">
-        <is>
-          <t>Naughty</t>
-        </is>
-      </c>
+          <t>Isl</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" t="n">
-        <v>922597</v>
+        <v>631716</v>
       </c>
       <c r="B100" t="inlineStr">
         <is>
@@ -2564,7 +2564,7 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>Girl</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
@@ -2572,15 +2572,11 @@
           <t>Msc</t>
         </is>
       </c>
-      <c r="E100" t="inlineStr">
-        <is>
-          <t>Naughty</t>
-        </is>
-      </c>
+      <c r="E100" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" t="n">
-        <v>123701</v>
+        <v>958502</v>
       </c>
       <c r="B101" t="inlineStr">
         <is>
@@ -2589,7 +2585,7 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>Girl</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
@@ -2601,7 +2597,7 @@
     </row>
     <row r="102">
       <c r="A102" t="n">
-        <v>672348</v>
+        <v>770007</v>
       </c>
       <c r="B102" t="inlineStr">
         <is>
@@ -2610,19 +2606,19 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>Boy</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>Msc</t>
+          <t>Isl</t>
         </is>
       </c>
       <c r="E102" t="inlineStr"/>
     </row>
     <row r="103">
       <c r="A103" t="n">
-        <v>231099</v>
+        <v>816671</v>
       </c>
       <c r="B103" t="inlineStr">
         <is>
@@ -2631,7 +2627,7 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>Girl</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
@@ -2643,7 +2639,7 @@
     </row>
     <row r="104">
       <c r="A104" t="n">
-        <v>374490</v>
+        <v>858020</v>
       </c>
       <c r="B104" t="inlineStr">
         <is>
@@ -2652,19 +2648,19 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>Boy</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>Isl</t>
+          <t>Msc</t>
         </is>
       </c>
       <c r="E104" t="inlineStr"/>
     </row>
     <row r="105">
       <c r="A105" t="n">
-        <v>999336</v>
+        <v>100808</v>
       </c>
       <c r="B105" t="inlineStr">
         <is>
@@ -2673,7 +2669,7 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>Boy</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
@@ -2685,7 +2681,7 @@
     </row>
     <row r="106">
       <c r="A106" t="n">
-        <v>363871</v>
+        <v>947317</v>
       </c>
       <c r="B106" t="inlineStr">
         <is>
@@ -2694,19 +2690,19 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>Girl</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>Msc</t>
+          <t>Isl</t>
         </is>
       </c>
       <c r="E106" t="inlineStr"/>
     </row>
     <row r="107">
       <c r="A107" t="n">
-        <v>396555</v>
+        <v>478843</v>
       </c>
       <c r="B107" t="inlineStr">
         <is>
@@ -2715,19 +2711,23 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>Boy</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>Msc</t>
-        </is>
-      </c>
-      <c r="E107" t="inlineStr"/>
+          <t>Isl</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>Naughty</t>
+        </is>
+      </c>
     </row>
     <row r="108">
       <c r="A108" t="n">
-        <v>524424</v>
+        <v>869557</v>
       </c>
       <c r="B108" t="inlineStr">
         <is>
@@ -2736,19 +2736,19 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>Girl</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>Msc</t>
+          <t>Isl</t>
         </is>
       </c>
       <c r="E108" t="inlineStr"/>
     </row>
     <row r="109">
       <c r="A109" t="n">
-        <v>228461</v>
+        <v>834849</v>
       </c>
       <c r="B109" t="inlineStr">
         <is>
@@ -2757,19 +2757,19 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>Boy</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>Msc</t>
+          <t>Isl</t>
         </is>
       </c>
       <c r="E109" t="inlineStr"/>
     </row>
     <row r="110">
       <c r="A110" t="n">
-        <v>541177</v>
+        <v>794334</v>
       </c>
       <c r="B110" t="inlineStr">
         <is>
@@ -2778,19 +2778,19 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>Girl</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>Msc</t>
+          <t>Isl</t>
         </is>
       </c>
       <c r="E110" t="inlineStr"/>
     </row>
     <row r="111">
       <c r="A111" t="n">
-        <v>129572</v>
+        <v>638525</v>
       </c>
       <c r="B111" t="inlineStr">
         <is>
@@ -2799,7 +2799,7 @@
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>Girl</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
@@ -2811,7 +2811,7 @@
     </row>
     <row r="112">
       <c r="A112" t="n">
-        <v>642481</v>
+        <v>853067</v>
       </c>
       <c r="B112" t="inlineStr">
         <is>
@@ -2820,7 +2820,7 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>Boy</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
@@ -2832,7 +2832,7 @@
     </row>
     <row r="113">
       <c r="A113" t="n">
-        <v>849724</v>
+        <v>103329</v>
       </c>
       <c r="B113" t="inlineStr">
         <is>
@@ -2841,19 +2841,19 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>Boy</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>Isl</t>
+          <t>Msc</t>
         </is>
       </c>
       <c r="E113" t="inlineStr"/>
     </row>
     <row r="114">
       <c r="A114" t="n">
-        <v>617254</v>
+        <v>665955</v>
       </c>
       <c r="B114" t="inlineStr">
         <is>
@@ -2862,7 +2862,7 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>Boy</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
@@ -2874,7 +2874,7 @@
     </row>
     <row r="115">
       <c r="A115" t="n">
-        <v>755232</v>
+        <v>288585</v>
       </c>
       <c r="B115" t="inlineStr">
         <is>
@@ -2883,7 +2883,7 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>Boy</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
@@ -2895,7 +2895,7 @@
     </row>
     <row r="116">
       <c r="A116" t="n">
-        <v>810199</v>
+        <v>349296</v>
       </c>
       <c r="B116" t="inlineStr">
         <is>
@@ -2904,7 +2904,7 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>Girl</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D116" t="inlineStr">
@@ -2916,7 +2916,7 @@
     </row>
     <row r="117">
       <c r="A117" t="n">
-        <v>742535</v>
+        <v>868351</v>
       </c>
       <c r="B117" t="inlineStr">
         <is>
@@ -2925,7 +2925,7 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>Girl</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
@@ -2937,7 +2937,7 @@
     </row>
     <row r="118">
       <c r="A118" t="n">
-        <v>690795</v>
+        <v>290870</v>
       </c>
       <c r="B118" t="inlineStr">
         <is>
@@ -2946,7 +2946,7 @@
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>Girl</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
@@ -2958,7 +2958,7 @@
     </row>
     <row r="119">
       <c r="A119" t="n">
-        <v>780722</v>
+        <v>242230</v>
       </c>
       <c r="B119" t="inlineStr">
         <is>
@@ -2967,7 +2967,7 @@
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>Boy</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D119" t="inlineStr">
@@ -2979,7 +2979,7 @@
     </row>
     <row r="120">
       <c r="A120" t="n">
-        <v>871381</v>
+        <v>241888</v>
       </c>
       <c r="B120" t="inlineStr">
         <is>
@@ -2988,23 +2988,19 @@
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>Boy</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>Isl</t>
-        </is>
-      </c>
-      <c r="E120" t="inlineStr">
-        <is>
-          <t>Naughty</t>
-        </is>
-      </c>
+          <t>Msc</t>
+        </is>
+      </c>
+      <c r="E120" t="inlineStr"/>
     </row>
     <row r="121">
       <c r="A121" t="n">
-        <v>127211</v>
+        <v>983334</v>
       </c>
       <c r="B121" t="inlineStr">
         <is>
@@ -3013,19 +3009,19 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>Girl</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>Msc</t>
+          <t>Isl</t>
         </is>
       </c>
       <c r="E121" t="inlineStr"/>
     </row>
     <row r="122">
       <c r="A122" t="n">
-        <v>391638</v>
+        <v>551203</v>
       </c>
       <c r="B122" t="inlineStr">
         <is>
@@ -3034,19 +3030,19 @@
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>Boy</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>Isl</t>
+          <t>Msc</t>
         </is>
       </c>
       <c r="E122" t="inlineStr"/>
     </row>
     <row r="123">
       <c r="A123" t="n">
-        <v>290109</v>
+        <v>644775</v>
       </c>
       <c r="B123" t="inlineStr">
         <is>
@@ -3055,19 +3051,19 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>Girl</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>Msc</t>
+          <t>Isl</t>
         </is>
       </c>
       <c r="E123" t="inlineStr"/>
     </row>
     <row r="124">
       <c r="A124" t="n">
-        <v>677384</v>
+        <v>915267</v>
       </c>
       <c r="B124" t="inlineStr">
         <is>
@@ -3076,19 +3072,19 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>Boy</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D124" t="inlineStr">
         <is>
-          <t>Msc</t>
+          <t>Isl</t>
         </is>
       </c>
       <c r="E124" t="inlineStr"/>
     </row>
     <row r="125">
       <c r="A125" t="n">
-        <v>297888</v>
+        <v>947104</v>
       </c>
       <c r="B125" t="inlineStr">
         <is>
@@ -3097,7 +3093,7 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>Boy</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D125" t="inlineStr">
@@ -3109,7 +3105,7 @@
     </row>
     <row r="126">
       <c r="A126" t="n">
-        <v>420420</v>
+        <v>179281</v>
       </c>
       <c r="B126" t="inlineStr">
         <is>
@@ -3118,7 +3114,7 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>Girl</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D126" t="inlineStr">
@@ -3130,7 +3126,7 @@
     </row>
     <row r="127">
       <c r="A127" t="n">
-        <v>598075</v>
+        <v>136397</v>
       </c>
       <c r="B127" t="inlineStr">
         <is>
@@ -3139,7 +3135,7 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>Boy</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D127" t="inlineStr">
@@ -3151,7 +3147,7 @@
     </row>
     <row r="128">
       <c r="A128" t="n">
-        <v>377877</v>
+        <v>911209</v>
       </c>
       <c r="B128" t="inlineStr">
         <is>
@@ -3160,19 +3156,19 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>Girl</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D128" t="inlineStr">
         <is>
-          <t>Isl</t>
+          <t>Msc</t>
         </is>
       </c>
       <c r="E128" t="inlineStr"/>
     </row>
     <row r="129">
       <c r="A129" t="n">
-        <v>517576</v>
+        <v>794049</v>
       </c>
       <c r="B129" t="inlineStr">
         <is>
@@ -3181,19 +3177,19 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>Girl</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t>Isl</t>
+          <t>Msc</t>
         </is>
       </c>
       <c r="E129" t="inlineStr"/>
     </row>
     <row r="130">
       <c r="A130" t="n">
-        <v>248949</v>
+        <v>795496</v>
       </c>
       <c r="B130" t="inlineStr">
         <is>
@@ -3202,19 +3198,23 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>Girl</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D130" t="inlineStr">
         <is>
-          <t>Isl</t>
-        </is>
-      </c>
-      <c r="E130" t="inlineStr"/>
+          <t>Msc</t>
+        </is>
+      </c>
+      <c r="E130" t="inlineStr">
+        <is>
+          <t>Weak in studies</t>
+        </is>
+      </c>
     </row>
     <row r="131">
       <c r="A131" t="n">
-        <v>153734</v>
+        <v>305910</v>
       </c>
       <c r="B131" t="inlineStr">
         <is>
@@ -3223,19 +3223,19 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>Boy</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D131" t="inlineStr">
         <is>
-          <t>Msc</t>
+          <t>Isl</t>
         </is>
       </c>
       <c r="E131" t="inlineStr"/>
     </row>
     <row r="132">
       <c r="A132" t="n">
-        <v>434329</v>
+        <v>210230</v>
       </c>
       <c r="B132" t="inlineStr">
         <is>
@@ -3244,7 +3244,7 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>Boy</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D132" t="inlineStr">
@@ -3256,7 +3256,7 @@
     </row>
     <row r="133">
       <c r="A133" t="n">
-        <v>925125</v>
+        <v>334791</v>
       </c>
       <c r="B133" t="inlineStr">
         <is>
@@ -3265,7 +3265,7 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>Boy</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D133" t="inlineStr">
@@ -3273,11 +3273,15 @@
           <t>Isl</t>
         </is>
       </c>
-      <c r="E133" t="inlineStr"/>
+      <c r="E133" t="inlineStr">
+        <is>
+          <t>Naughty</t>
+        </is>
+      </c>
     </row>
     <row r="134">
       <c r="A134" t="n">
-        <v>805866</v>
+        <v>124149</v>
       </c>
       <c r="B134" t="inlineStr">
         <is>
@@ -3286,7 +3290,7 @@
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>Girl</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D134" t="inlineStr">
@@ -3298,7 +3302,7 @@
     </row>
     <row r="135">
       <c r="A135" t="n">
-        <v>511013</v>
+        <v>432811</v>
       </c>
       <c r="B135" t="inlineStr">
         <is>
@@ -3307,7 +3311,7 @@
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>Girl</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D135" t="inlineStr">
@@ -3319,7 +3323,7 @@
     </row>
     <row r="136">
       <c r="A136" t="n">
-        <v>716508</v>
+        <v>636816</v>
       </c>
       <c r="B136" t="inlineStr">
         <is>
@@ -3328,19 +3332,19 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>Girl</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D136" t="inlineStr">
         <is>
-          <t>Isl</t>
+          <t>Msc</t>
         </is>
       </c>
       <c r="E136" t="inlineStr"/>
     </row>
     <row r="137">
       <c r="A137" t="n">
-        <v>339517</v>
+        <v>990284</v>
       </c>
       <c r="B137" t="inlineStr">
         <is>
@@ -3349,7 +3353,7 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>Girl</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D137" t="inlineStr">
@@ -3361,7 +3365,7 @@
     </row>
     <row r="138">
       <c r="A138" t="n">
-        <v>133794</v>
+        <v>516400</v>
       </c>
       <c r="B138" t="inlineStr">
         <is>
@@ -3370,19 +3374,19 @@
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>Girl</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D138" t="inlineStr">
         <is>
-          <t>Msc</t>
+          <t>Isl</t>
         </is>
       </c>
       <c r="E138" t="inlineStr"/>
     </row>
     <row r="139">
       <c r="A139" t="n">
-        <v>860228</v>
+        <v>778043</v>
       </c>
       <c r="B139" t="inlineStr">
         <is>
@@ -3391,7 +3395,7 @@
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>Girl</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D139" t="inlineStr">
@@ -3403,7 +3407,7 @@
     </row>
     <row r="140">
       <c r="A140" t="n">
-        <v>870224</v>
+        <v>204471</v>
       </c>
       <c r="B140" t="inlineStr">
         <is>
@@ -3412,19 +3416,19 @@
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>Boy</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D140" t="inlineStr">
         <is>
-          <t>Msc</t>
+          <t>Isl</t>
         </is>
       </c>
       <c r="E140" t="inlineStr"/>
     </row>
     <row r="141">
       <c r="A141" t="n">
-        <v>450254</v>
+        <v>179109</v>
       </c>
       <c r="B141" t="inlineStr">
         <is>
@@ -3433,7 +3437,7 @@
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>Girl</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D141" t="inlineStr">
@@ -3445,7 +3449,7 @@
     </row>
     <row r="142">
       <c r="A142" t="n">
-        <v>236368</v>
+        <v>776595</v>
       </c>
       <c r="B142" t="inlineStr">
         <is>
@@ -3454,19 +3458,19 @@
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>Boy</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D142" t="inlineStr">
         <is>
-          <t>Isl</t>
+          <t>Msc</t>
         </is>
       </c>
       <c r="E142" t="inlineStr"/>
     </row>
     <row r="143">
       <c r="A143" t="n">
-        <v>513870</v>
+        <v>281942</v>
       </c>
       <c r="B143" t="inlineStr">
         <is>
@@ -3475,19 +3479,19 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>Girl</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D143" t="inlineStr">
         <is>
-          <t>Msc</t>
+          <t>Isl</t>
         </is>
       </c>
       <c r="E143" t="inlineStr"/>
     </row>
     <row r="144">
       <c r="A144" t="n">
-        <v>417082</v>
+        <v>530758</v>
       </c>
       <c r="B144" t="inlineStr">
         <is>
@@ -3496,19 +3500,19 @@
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>Boy</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D144" t="inlineStr">
         <is>
-          <t>Isl</t>
+          <t>Msc</t>
         </is>
       </c>
       <c r="E144" t="inlineStr"/>
     </row>
     <row r="145">
       <c r="A145" t="n">
-        <v>401895</v>
+        <v>827035</v>
       </c>
       <c r="B145" t="inlineStr">
         <is>
@@ -3517,7 +3521,7 @@
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>Boy</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D145" t="inlineStr">
@@ -3529,7 +3533,7 @@
     </row>
     <row r="146">
       <c r="A146" t="n">
-        <v>913418</v>
+        <v>226372</v>
       </c>
       <c r="B146" t="inlineStr">
         <is>
@@ -3538,19 +3542,19 @@
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>Girl</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D146" t="inlineStr">
         <is>
-          <t>Msc</t>
+          <t>Isl</t>
         </is>
       </c>
       <c r="E146" t="inlineStr"/>
     </row>
     <row r="147">
       <c r="A147" t="n">
-        <v>572362</v>
+        <v>995976</v>
       </c>
       <c r="B147" t="inlineStr">
         <is>
@@ -3559,23 +3563,19 @@
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>Girl</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D147" t="inlineStr">
         <is>
-          <t>Msc</t>
-        </is>
-      </c>
-      <c r="E147" t="inlineStr">
-        <is>
-          <t>Naughty</t>
-        </is>
-      </c>
+          <t>Isl</t>
+        </is>
+      </c>
+      <c r="E147" t="inlineStr"/>
     </row>
     <row r="148">
       <c r="A148" t="n">
-        <v>751678</v>
+        <v>990771</v>
       </c>
       <c r="B148" t="inlineStr">
         <is>
@@ -3584,7 +3584,7 @@
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>Boy</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D148" t="inlineStr">
@@ -3596,7 +3596,7 @@
     </row>
     <row r="149">
       <c r="A149" t="n">
-        <v>920452</v>
+        <v>640630</v>
       </c>
       <c r="B149" t="inlineStr">
         <is>
@@ -3605,23 +3605,19 @@
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>Boy</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D149" t="inlineStr">
         <is>
-          <t>Isl</t>
-        </is>
-      </c>
-      <c r="E149" t="inlineStr">
-        <is>
-          <t>Naughty</t>
-        </is>
-      </c>
+          <t>Msc</t>
+        </is>
+      </c>
+      <c r="E149" t="inlineStr"/>
     </row>
     <row r="150">
       <c r="A150" t="n">
-        <v>956087</v>
+        <v>623403</v>
       </c>
       <c r="B150" t="inlineStr">
         <is>
@@ -3630,19 +3626,19 @@
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>Girl</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D150" t="inlineStr">
         <is>
-          <t>Msc</t>
+          <t>Isl</t>
         </is>
       </c>
       <c r="E150" t="inlineStr"/>
     </row>
     <row r="151">
       <c r="A151" t="n">
-        <v>101419</v>
+        <v>314203</v>
       </c>
       <c r="B151" t="inlineStr">
         <is>
@@ -3651,7 +3647,7 @@
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>Girl</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D151" t="inlineStr">
@@ -3663,7 +3659,7 @@
     </row>
     <row r="152">
       <c r="A152" t="n">
-        <v>689816</v>
+        <v>114494</v>
       </c>
       <c r="B152" t="inlineStr">
         <is>
@@ -3672,19 +3668,19 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>Girl</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D152" t="inlineStr">
         <is>
-          <t>Isl</t>
+          <t>Msc</t>
         </is>
       </c>
       <c r="E152" t="inlineStr"/>
     </row>
     <row r="153">
       <c r="A153" t="n">
-        <v>372073</v>
+        <v>713088</v>
       </c>
       <c r="B153" t="inlineStr">
         <is>
@@ -3693,7 +3689,7 @@
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>Girl</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D153" t="inlineStr">
@@ -3705,7 +3701,7 @@
     </row>
     <row r="154">
       <c r="A154" t="n">
-        <v>546500</v>
+        <v>836599</v>
       </c>
       <c r="B154" t="inlineStr">
         <is>
@@ -3714,19 +3710,19 @@
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>Boy</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D154" t="inlineStr">
         <is>
-          <t>Isl</t>
+          <t>Msc</t>
         </is>
       </c>
       <c r="E154" t="inlineStr"/>
     </row>
     <row r="155">
       <c r="A155" t="n">
-        <v>696335</v>
+        <v>576946</v>
       </c>
       <c r="B155" t="inlineStr">
         <is>
@@ -3735,7 +3731,7 @@
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>Girl</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D155" t="inlineStr">
@@ -3747,7 +3743,7 @@
     </row>
     <row r="156">
       <c r="A156" t="n">
-        <v>199509</v>
+        <v>199333</v>
       </c>
       <c r="B156" t="inlineStr">
         <is>
@@ -3756,7 +3752,7 @@
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>Girl</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D156" t="inlineStr">
@@ -3768,7 +3764,7 @@
     </row>
     <row r="157">
       <c r="A157" t="n">
-        <v>881364</v>
+        <v>504651</v>
       </c>
       <c r="B157" t="inlineStr">
         <is>
@@ -3777,7 +3773,7 @@
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>Boy</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D157" t="inlineStr">
@@ -3789,7 +3785,7 @@
     </row>
     <row r="158">
       <c r="A158" t="n">
-        <v>661936</v>
+        <v>245979</v>
       </c>
       <c r="B158" t="inlineStr">
         <is>
@@ -3798,7 +3794,7 @@
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>Girl</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D158" t="inlineStr">
@@ -3810,7 +3806,7 @@
     </row>
     <row r="159">
       <c r="A159" t="n">
-        <v>873050</v>
+        <v>156038</v>
       </c>
       <c r="B159" t="inlineStr">
         <is>
@@ -3819,7 +3815,7 @@
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>Boy</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D159" t="inlineStr">
@@ -3831,7 +3827,7 @@
     </row>
     <row r="160">
       <c r="A160" t="n">
-        <v>662717</v>
+        <v>207017</v>
       </c>
       <c r="B160" t="inlineStr">
         <is>
@@ -3840,19 +3836,19 @@
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>Girl</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D160" t="inlineStr">
         <is>
-          <t>Isl</t>
+          <t>Msc</t>
         </is>
       </c>
       <c r="E160" t="inlineStr"/>
     </row>
     <row r="161">
       <c r="A161" t="n">
-        <v>196229</v>
+        <v>821697</v>
       </c>
       <c r="B161" t="inlineStr">
         <is>
@@ -3861,7 +3857,7 @@
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>Boy</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D161" t="inlineStr">
@@ -3873,7 +3869,7 @@
     </row>
     <row r="162">
       <c r="A162" t="n">
-        <v>390896</v>
+        <v>380867</v>
       </c>
       <c r="B162" t="inlineStr">
         <is>
@@ -3882,19 +3878,19 @@
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>Girl</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D162" t="inlineStr">
         <is>
-          <t>Isl</t>
+          <t>Msc</t>
         </is>
       </c>
       <c r="E162" t="inlineStr"/>
     </row>
     <row r="163">
       <c r="A163" t="n">
-        <v>641925</v>
+        <v>889998</v>
       </c>
       <c r="B163" t="inlineStr">
         <is>
@@ -3903,19 +3899,19 @@
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>Girl</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D163" t="inlineStr">
         <is>
-          <t>Msc</t>
+          <t>Isl</t>
         </is>
       </c>
       <c r="E163" t="inlineStr"/>
     </row>
     <row r="164">
       <c r="A164" t="n">
-        <v>269884</v>
+        <v>769589</v>
       </c>
       <c r="B164" t="inlineStr">
         <is>
@@ -3924,19 +3920,19 @@
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>Boy</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D164" t="inlineStr">
         <is>
-          <t>Isl</t>
+          <t>Msc</t>
         </is>
       </c>
       <c r="E164" t="inlineStr"/>
     </row>
     <row r="165">
       <c r="A165" t="n">
-        <v>571817</v>
+        <v>106884</v>
       </c>
       <c r="B165" t="inlineStr">
         <is>
@@ -3945,19 +3941,19 @@
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>Boy</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D165" t="inlineStr">
         <is>
-          <t>Msc</t>
+          <t>Isl</t>
         </is>
       </c>
       <c r="E165" t="inlineStr"/>
     </row>
     <row r="166">
       <c r="A166" t="n">
-        <v>864030</v>
+        <v>197478</v>
       </c>
       <c r="B166" t="inlineStr">
         <is>
@@ -3966,7 +3962,7 @@
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>Girl</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D166" t="inlineStr">
@@ -3978,7 +3974,7 @@
     </row>
     <row r="167">
       <c r="A167" t="n">
-        <v>353570</v>
+        <v>350329</v>
       </c>
       <c r="B167" t="inlineStr">
         <is>
@@ -3987,7 +3983,7 @@
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>Boy</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D167" t="inlineStr">
@@ -3999,7 +3995,7 @@
     </row>
     <row r="168">
       <c r="A168" t="n">
-        <v>672897</v>
+        <v>270592</v>
       </c>
       <c r="B168" t="inlineStr">
         <is>
@@ -4008,7 +4004,7 @@
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>Girl</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D168" t="inlineStr">
@@ -4020,7 +4016,7 @@
     </row>
     <row r="169">
       <c r="A169" t="n">
-        <v>868485</v>
+        <v>843959</v>
       </c>
       <c r="B169" t="inlineStr">
         <is>
@@ -4029,7 +4025,7 @@
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>Boy</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D169" t="inlineStr">
@@ -4041,7 +4037,7 @@
     </row>
     <row r="170">
       <c r="A170" t="n">
-        <v>834259</v>
+        <v>622498</v>
       </c>
       <c r="B170" t="inlineStr">
         <is>
@@ -4050,7 +4046,7 @@
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>Girl</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D170" t="inlineStr">
@@ -4062,7 +4058,7 @@
     </row>
     <row r="171">
       <c r="A171" t="n">
-        <v>563933</v>
+        <v>921465</v>
       </c>
       <c r="B171" t="inlineStr">
         <is>
@@ -4071,19 +4067,19 @@
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>Boy</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D171" t="inlineStr">
         <is>
-          <t>Msc</t>
+          <t>Isl</t>
         </is>
       </c>
       <c r="E171" t="inlineStr"/>
     </row>
     <row r="172">
       <c r="A172" t="n">
-        <v>443074</v>
+        <v>782149</v>
       </c>
       <c r="B172" t="inlineStr">
         <is>
@@ -4092,7 +4088,7 @@
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>Girl</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D172" t="inlineStr">
@@ -4104,7 +4100,7 @@
     </row>
     <row r="173">
       <c r="A173" t="n">
-        <v>494701</v>
+        <v>116890</v>
       </c>
       <c r="B173" t="inlineStr">
         <is>
@@ -4113,19 +4109,19 @@
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>Girl</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D173" t="inlineStr">
         <is>
-          <t>Isl</t>
+          <t>Msc</t>
         </is>
       </c>
       <c r="E173" t="inlineStr"/>
     </row>
     <row r="174">
       <c r="A174" t="n">
-        <v>988687</v>
+        <v>192648</v>
       </c>
       <c r="B174" t="inlineStr">
         <is>
@@ -4134,7 +4130,7 @@
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>Boy</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D174" t="inlineStr">
@@ -4146,7 +4142,7 @@
     </row>
     <row r="175">
       <c r="A175" t="n">
-        <v>485385</v>
+        <v>895720</v>
       </c>
       <c r="B175" t="inlineStr">
         <is>
@@ -4155,7 +4151,7 @@
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>Girl</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D175" t="inlineStr">
@@ -4167,7 +4163,7 @@
     </row>
     <row r="176">
       <c r="A176" t="n">
-        <v>299460</v>
+        <v>654396</v>
       </c>
       <c r="B176" t="inlineStr">
         <is>
@@ -4176,7 +4172,7 @@
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>Boy</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D176" t="inlineStr">
@@ -4188,7 +4184,7 @@
     </row>
     <row r="177">
       <c r="A177" t="n">
-        <v>712357</v>
+        <v>787226</v>
       </c>
       <c r="B177" t="inlineStr">
         <is>
@@ -4197,19 +4193,19 @@
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>Boy</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D177" t="inlineStr">
         <is>
-          <t>Msc</t>
+          <t>Isl</t>
         </is>
       </c>
       <c r="E177" t="inlineStr"/>
     </row>
     <row r="178">
       <c r="A178" t="n">
-        <v>522368</v>
+        <v>318843</v>
       </c>
       <c r="B178" t="inlineStr">
         <is>
@@ -4218,19 +4214,19 @@
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>Boy</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D178" t="inlineStr">
         <is>
-          <t>Isl</t>
+          <t>Msc</t>
         </is>
       </c>
       <c r="E178" t="inlineStr"/>
     </row>
     <row r="179">
       <c r="A179" t="n">
-        <v>299431</v>
+        <v>164101</v>
       </c>
       <c r="B179" t="inlineStr">
         <is>
@@ -4239,7 +4235,7 @@
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>Boy</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D179" t="inlineStr">
@@ -4251,7 +4247,7 @@
     </row>
     <row r="180">
       <c r="A180" t="n">
-        <v>876384</v>
+        <v>988188</v>
       </c>
       <c r="B180" t="inlineStr">
         <is>
@@ -4260,19 +4256,19 @@
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>Boy</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D180" t="inlineStr">
         <is>
-          <t>Msc</t>
+          <t>Isl</t>
         </is>
       </c>
       <c r="E180" t="inlineStr"/>
     </row>
     <row r="181">
       <c r="A181" t="n">
-        <v>982732</v>
+        <v>353272</v>
       </c>
       <c r="B181" t="inlineStr">
         <is>
@@ -4281,19 +4277,19 @@
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>Boy</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D181" t="inlineStr">
         <is>
-          <t>Msc</t>
+          <t>Isl</t>
         </is>
       </c>
       <c r="E181" t="inlineStr"/>
     </row>
     <row r="182">
       <c r="A182" t="n">
-        <v>790420</v>
+        <v>611577</v>
       </c>
       <c r="B182" t="inlineStr">
         <is>
@@ -4302,7 +4298,7 @@
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>Boy</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D182" t="inlineStr">
@@ -4314,7 +4310,7 @@
     </row>
     <row r="183">
       <c r="A183" t="n">
-        <v>381683</v>
+        <v>613486</v>
       </c>
       <c r="B183" t="inlineStr">
         <is>
@@ -4323,19 +4319,19 @@
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>Girl</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D183" t="inlineStr">
         <is>
-          <t>Isl</t>
+          <t>Msc</t>
         </is>
       </c>
       <c r="E183" t="inlineStr"/>
     </row>
     <row r="184">
       <c r="A184" t="n">
-        <v>916304</v>
+        <v>113856</v>
       </c>
       <c r="B184" t="inlineStr">
         <is>
@@ -4344,7 +4340,7 @@
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>Boy</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D184" t="inlineStr">
@@ -4352,11 +4348,15 @@
           <t>Isl</t>
         </is>
       </c>
-      <c r="E184" t="inlineStr"/>
+      <c r="E184" t="inlineStr">
+        <is>
+          <t>Naughty</t>
+        </is>
+      </c>
     </row>
     <row r="185">
       <c r="A185" t="n">
-        <v>787072</v>
+        <v>716906</v>
       </c>
       <c r="B185" t="inlineStr">
         <is>
@@ -4365,7 +4365,7 @@
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>Girl</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D185" t="inlineStr">
@@ -4377,7 +4377,7 @@
     </row>
     <row r="186">
       <c r="A186" t="n">
-        <v>684180</v>
+        <v>486066</v>
       </c>
       <c r="B186" t="inlineStr">
         <is>
@@ -4386,7 +4386,7 @@
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>Boy</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D186" t="inlineStr">
@@ -4398,7 +4398,7 @@
     </row>
     <row r="187">
       <c r="A187" t="n">
-        <v>335227</v>
+        <v>842790</v>
       </c>
       <c r="B187" t="inlineStr">
         <is>
@@ -4407,19 +4407,19 @@
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>Boy</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D187" t="inlineStr">
         <is>
-          <t>Isl</t>
+          <t>Msc</t>
         </is>
       </c>
       <c r="E187" t="inlineStr"/>
     </row>
     <row r="188">
       <c r="A188" t="n">
-        <v>244757</v>
+        <v>844589</v>
       </c>
       <c r="B188" t="inlineStr">
         <is>
@@ -4428,7 +4428,7 @@
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>Girl</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D188" t="inlineStr">
@@ -4440,7 +4440,7 @@
     </row>
     <row r="189">
       <c r="A189" t="n">
-        <v>465606</v>
+        <v>202062</v>
       </c>
       <c r="B189" t="inlineStr">
         <is>
@@ -4449,19 +4449,23 @@
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>Girl</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D189" t="inlineStr">
         <is>
-          <t>Msc</t>
-        </is>
-      </c>
-      <c r="E189" t="inlineStr"/>
+          <t>Isl</t>
+        </is>
+      </c>
+      <c r="E189" t="inlineStr">
+        <is>
+          <t>Weak in studies</t>
+        </is>
+      </c>
     </row>
     <row r="190">
       <c r="A190" t="n">
-        <v>701007</v>
+        <v>791430</v>
       </c>
       <c r="B190" t="inlineStr">
         <is>
@@ -4470,19 +4474,19 @@
       </c>
       <c r="C190" t="inlineStr">
         <is>
-          <t>Boy</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D190" t="inlineStr">
         <is>
-          <t>Isl</t>
+          <t>Msc</t>
         </is>
       </c>
       <c r="E190" t="inlineStr"/>
     </row>
     <row r="191">
       <c r="A191" t="n">
-        <v>688177</v>
+        <v>860054</v>
       </c>
       <c r="B191" t="inlineStr">
         <is>
@@ -4491,19 +4495,19 @@
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>Girl</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D191" t="inlineStr">
         <is>
-          <t>Isl</t>
+          <t>Msc</t>
         </is>
       </c>
       <c r="E191" t="inlineStr"/>
     </row>
     <row r="192">
       <c r="A192" t="n">
-        <v>102328</v>
+        <v>597905</v>
       </c>
       <c r="B192" t="inlineStr">
         <is>
@@ -4512,19 +4516,23 @@
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>Girl</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D192" t="inlineStr">
         <is>
-          <t>Msc</t>
-        </is>
-      </c>
-      <c r="E192" t="inlineStr"/>
+          <t>Isl</t>
+        </is>
+      </c>
+      <c r="E192" t="inlineStr">
+        <is>
+          <t>Weak in studies</t>
+        </is>
+      </c>
     </row>
     <row r="193">
       <c r="A193" t="n">
-        <v>481260</v>
+        <v>125722</v>
       </c>
       <c r="B193" t="inlineStr">
         <is>
@@ -4533,7 +4541,7 @@
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>Girl</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D193" t="inlineStr">
@@ -4545,7 +4553,7 @@
     </row>
     <row r="194">
       <c r="A194" t="n">
-        <v>994179</v>
+        <v>383887</v>
       </c>
       <c r="B194" t="inlineStr">
         <is>
@@ -4554,19 +4562,19 @@
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>Boy</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D194" t="inlineStr">
         <is>
-          <t>Isl</t>
+          <t>Msc</t>
         </is>
       </c>
       <c r="E194" t="inlineStr"/>
     </row>
     <row r="195">
       <c r="A195" t="n">
-        <v>897008</v>
+        <v>732328</v>
       </c>
       <c r="B195" t="inlineStr">
         <is>
@@ -4575,19 +4583,19 @@
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>Girl</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D195" t="inlineStr">
         <is>
-          <t>Msc</t>
+          <t>Isl</t>
         </is>
       </c>
       <c r="E195" t="inlineStr"/>
     </row>
     <row r="196">
       <c r="A196" t="n">
-        <v>609045</v>
+        <v>872994</v>
       </c>
       <c r="B196" t="inlineStr">
         <is>
@@ -4596,7 +4604,7 @@
       </c>
       <c r="C196" t="inlineStr">
         <is>
-          <t>Boy</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D196" t="inlineStr">
@@ -4608,7 +4616,7 @@
     </row>
     <row r="197">
       <c r="A197" t="n">
-        <v>206936</v>
+        <v>676692</v>
       </c>
       <c r="B197" t="inlineStr">
         <is>
@@ -4617,7 +4625,7 @@
       </c>
       <c r="C197" t="inlineStr">
         <is>
-          <t>Boy</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D197" t="inlineStr">
@@ -4629,7 +4637,7 @@
     </row>
     <row r="198">
       <c r="A198" t="n">
-        <v>298624</v>
+        <v>442300</v>
       </c>
       <c r="B198" t="inlineStr">
         <is>
@@ -4638,7 +4646,7 @@
       </c>
       <c r="C198" t="inlineStr">
         <is>
-          <t>Girl</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D198" t="inlineStr">
@@ -4650,7 +4658,7 @@
     </row>
     <row r="199">
       <c r="A199" t="n">
-        <v>499690</v>
+        <v>869162</v>
       </c>
       <c r="B199" t="inlineStr">
         <is>
@@ -4659,23 +4667,19 @@
       </c>
       <c r="C199" t="inlineStr">
         <is>
-          <t>Boy</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D199" t="inlineStr">
         <is>
-          <t>Isl</t>
-        </is>
-      </c>
-      <c r="E199" t="inlineStr">
-        <is>
-          <t>Naughty</t>
-        </is>
-      </c>
+          <t>Msc</t>
+        </is>
+      </c>
+      <c r="E199" t="inlineStr"/>
     </row>
     <row r="200">
       <c r="A200" t="n">
-        <v>935898</v>
+        <v>257343</v>
       </c>
       <c r="B200" t="inlineStr">
         <is>
@@ -4684,7 +4688,7 @@
       </c>
       <c r="C200" t="inlineStr">
         <is>
-          <t>Girl</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D200" t="inlineStr">
@@ -4696,7 +4700,7 @@
     </row>
     <row r="201">
       <c r="A201" t="n">
-        <v>111310</v>
+        <v>672651</v>
       </c>
       <c r="B201" t="inlineStr">
         <is>
@@ -4705,7 +4709,7 @@
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>Girl</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D201" t="inlineStr">
@@ -4717,7 +4721,7 @@
     </row>
     <row r="202">
       <c r="A202" t="n">
-        <v>572930</v>
+        <v>952198</v>
       </c>
       <c r="B202" t="inlineStr">
         <is>
@@ -4726,7 +4730,7 @@
       </c>
       <c r="C202" t="inlineStr">
         <is>
-          <t>Boy</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D202" t="inlineStr">
@@ -4738,7 +4742,7 @@
     </row>
     <row r="203">
       <c r="A203" t="n">
-        <v>562921</v>
+        <v>866290</v>
       </c>
       <c r="B203" t="inlineStr">
         <is>
@@ -4747,7 +4751,7 @@
       </c>
       <c r="C203" t="inlineStr">
         <is>
-          <t>Boy</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D203" t="inlineStr">
@@ -4759,7 +4763,7 @@
     </row>
     <row r="204">
       <c r="A204" t="n">
-        <v>970230</v>
+        <v>973268</v>
       </c>
       <c r="B204" t="inlineStr">
         <is>
@@ -4768,7 +4772,7 @@
       </c>
       <c r="C204" t="inlineStr">
         <is>
-          <t>Girl</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D204" t="inlineStr">
@@ -4780,7 +4784,7 @@
     </row>
     <row r="205">
       <c r="A205" t="n">
-        <v>711171</v>
+        <v>707657</v>
       </c>
       <c r="B205" t="inlineStr">
         <is>
@@ -4789,19 +4793,19 @@
       </c>
       <c r="C205" t="inlineStr">
         <is>
-          <t>Boy</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D205" t="inlineStr">
         <is>
-          <t>Isl</t>
+          <t>Msc</t>
         </is>
       </c>
       <c r="E205" t="inlineStr"/>
     </row>
     <row r="206">
       <c r="A206" t="n">
-        <v>791201</v>
+        <v>222902</v>
       </c>
       <c r="B206" t="inlineStr">
         <is>
@@ -4810,7 +4814,7 @@
       </c>
       <c r="C206" t="inlineStr">
         <is>
-          <t>Boy</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D206" t="inlineStr">
@@ -4818,15 +4822,11 @@
           <t>Isl</t>
         </is>
       </c>
-      <c r="E206" t="inlineStr">
-        <is>
-          <t>Weak in studies</t>
-        </is>
-      </c>
+      <c r="E206" t="inlineStr"/>
     </row>
     <row r="207">
       <c r="A207" t="n">
-        <v>443594</v>
+        <v>328330</v>
       </c>
       <c r="B207" t="inlineStr">
         <is>
@@ -4835,7 +4835,7 @@
       </c>
       <c r="C207" t="inlineStr">
         <is>
-          <t>Girl</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D207" t="inlineStr">
@@ -4847,7 +4847,7 @@
     </row>
     <row r="208">
       <c r="A208" t="n">
-        <v>999923</v>
+        <v>299729</v>
       </c>
       <c r="B208" t="inlineStr">
         <is>
@@ -4856,7 +4856,7 @@
       </c>
       <c r="C208" t="inlineStr">
         <is>
-          <t>Girl</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D208" t="inlineStr">
@@ -4868,7 +4868,7 @@
     </row>
     <row r="209">
       <c r="A209" t="n">
-        <v>248563</v>
+        <v>102486</v>
       </c>
       <c r="B209" t="inlineStr">
         <is>
@@ -4877,19 +4877,19 @@
       </c>
       <c r="C209" t="inlineStr">
         <is>
-          <t>Boy</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D209" t="inlineStr">
         <is>
-          <t>Isl</t>
+          <t>Msc</t>
         </is>
       </c>
       <c r="E209" t="inlineStr"/>
     </row>
     <row r="210">
       <c r="A210" t="n">
-        <v>631884</v>
+        <v>397077</v>
       </c>
       <c r="B210" t="inlineStr">
         <is>
@@ -4898,7 +4898,7 @@
       </c>
       <c r="C210" t="inlineStr">
         <is>
-          <t>Boy</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D210" t="inlineStr">
@@ -4910,7 +4910,7 @@
     </row>
     <row r="211">
       <c r="A211" t="n">
-        <v>526624</v>
+        <v>762964</v>
       </c>
       <c r="B211" t="inlineStr">
         <is>
@@ -4919,7 +4919,7 @@
       </c>
       <c r="C211" t="inlineStr">
         <is>
-          <t>Girl</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D211" t="inlineStr">
@@ -4931,7 +4931,7 @@
     </row>
     <row r="212">
       <c r="A212" t="n">
-        <v>581200</v>
+        <v>635051</v>
       </c>
       <c r="B212" t="inlineStr">
         <is>
@@ -4940,7 +4940,7 @@
       </c>
       <c r="C212" t="inlineStr">
         <is>
-          <t>Girl</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D212" t="inlineStr">
@@ -4952,7 +4952,7 @@
     </row>
     <row r="213">
       <c r="A213" t="n">
-        <v>529292</v>
+        <v>736173</v>
       </c>
       <c r="B213" t="inlineStr">
         <is>
@@ -4961,7 +4961,7 @@
       </c>
       <c r="C213" t="inlineStr">
         <is>
-          <t>Boy</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D213" t="inlineStr">
@@ -4973,7 +4973,7 @@
     </row>
     <row r="214">
       <c r="A214" t="n">
-        <v>106999</v>
+        <v>799937</v>
       </c>
       <c r="B214" t="inlineStr">
         <is>
@@ -4982,7 +4982,7 @@
       </c>
       <c r="C214" t="inlineStr">
         <is>
-          <t>Boy</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D214" t="inlineStr">
@@ -4994,7 +4994,7 @@
     </row>
     <row r="215">
       <c r="A215" t="n">
-        <v>727209</v>
+        <v>783822</v>
       </c>
       <c r="B215" t="inlineStr">
         <is>
@@ -5003,7 +5003,7 @@
       </c>
       <c r="C215" t="inlineStr">
         <is>
-          <t>Girl</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D215" t="inlineStr">
@@ -5015,7 +5015,7 @@
     </row>
     <row r="216">
       <c r="A216" t="n">
-        <v>617087</v>
+        <v>212203</v>
       </c>
       <c r="B216" t="inlineStr">
         <is>
@@ -5024,19 +5024,19 @@
       </c>
       <c r="C216" t="inlineStr">
         <is>
-          <t>Boy</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D216" t="inlineStr">
         <is>
-          <t>Isl</t>
+          <t>Msc</t>
         </is>
       </c>
       <c r="E216" t="inlineStr"/>
     </row>
     <row r="217">
       <c r="A217" t="n">
-        <v>885798</v>
+        <v>886022</v>
       </c>
       <c r="B217" t="inlineStr">
         <is>
@@ -5045,19 +5045,19 @@
       </c>
       <c r="C217" t="inlineStr">
         <is>
-          <t>Boy</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D217" t="inlineStr">
         <is>
-          <t>Msc</t>
+          <t>Isl</t>
         </is>
       </c>
       <c r="E217" t="inlineStr"/>
     </row>
     <row r="218">
       <c r="A218" t="n">
-        <v>453471</v>
+        <v>865953</v>
       </c>
       <c r="B218" t="inlineStr">
         <is>
@@ -5066,7 +5066,7 @@
       </c>
       <c r="C218" t="inlineStr">
         <is>
-          <t>Boy</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D218" t="inlineStr">
@@ -5078,7 +5078,7 @@
     </row>
     <row r="219">
       <c r="A219" t="n">
-        <v>928660</v>
+        <v>541391</v>
       </c>
       <c r="B219" t="inlineStr">
         <is>
@@ -5087,7 +5087,7 @@
       </c>
       <c r="C219" t="inlineStr">
         <is>
-          <t>Girl</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D219" t="inlineStr">
@@ -5099,7 +5099,7 @@
     </row>
     <row r="220">
       <c r="A220" t="n">
-        <v>708102</v>
+        <v>993257</v>
       </c>
       <c r="B220" t="inlineStr">
         <is>
@@ -5108,19 +5108,19 @@
       </c>
       <c r="C220" t="inlineStr">
         <is>
-          <t>Boy</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D220" t="inlineStr">
         <is>
-          <t>Isl</t>
+          <t>Msc</t>
         </is>
       </c>
       <c r="E220" t="inlineStr"/>
     </row>
     <row r="221">
       <c r="A221" t="n">
-        <v>626041</v>
+        <v>515105</v>
       </c>
       <c r="B221" t="inlineStr">
         <is>
@@ -5129,7 +5129,7 @@
       </c>
       <c r="C221" t="inlineStr">
         <is>
-          <t>Boy</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D221" t="inlineStr">
@@ -5141,7 +5141,7 @@
     </row>
     <row r="222">
       <c r="A222" t="n">
-        <v>793277</v>
+        <v>709207</v>
       </c>
       <c r="B222" t="inlineStr">
         <is>
@@ -5150,19 +5150,19 @@
       </c>
       <c r="C222" t="inlineStr">
         <is>
-          <t>Boy</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D222" t="inlineStr">
         <is>
-          <t>Msc</t>
+          <t>Isl</t>
         </is>
       </c>
       <c r="E222" t="inlineStr"/>
     </row>
     <row r="223">
       <c r="A223" t="n">
-        <v>872427</v>
+        <v>811651</v>
       </c>
       <c r="B223" t="inlineStr">
         <is>
@@ -5171,19 +5171,19 @@
       </c>
       <c r="C223" t="inlineStr">
         <is>
-          <t>Boy</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D223" t="inlineStr">
         <is>
-          <t>Msc</t>
+          <t>Isl</t>
         </is>
       </c>
       <c r="E223" t="inlineStr"/>
     </row>
     <row r="224">
       <c r="A224" t="n">
-        <v>879342</v>
+        <v>899577</v>
       </c>
       <c r="B224" t="inlineStr">
         <is>
@@ -5192,7 +5192,7 @@
       </c>
       <c r="C224" t="inlineStr">
         <is>
-          <t>Boy</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D224" t="inlineStr">
@@ -5200,11 +5200,15 @@
           <t>Msc</t>
         </is>
       </c>
-      <c r="E224" t="inlineStr"/>
+      <c r="E224" t="inlineStr">
+        <is>
+          <t>Naughty</t>
+        </is>
+      </c>
     </row>
     <row r="225">
       <c r="A225" t="n">
-        <v>828226</v>
+        <v>519569</v>
       </c>
       <c r="B225" t="inlineStr">
         <is>
@@ -5213,19 +5217,19 @@
       </c>
       <c r="C225" t="inlineStr">
         <is>
-          <t>Boy</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D225" t="inlineStr">
         <is>
-          <t>Isl</t>
+          <t>Msc</t>
         </is>
       </c>
       <c r="E225" t="inlineStr"/>
     </row>
     <row r="226">
       <c r="A226" t="n">
-        <v>485167</v>
+        <v>570099</v>
       </c>
       <c r="B226" t="inlineStr">
         <is>
@@ -5234,7 +5238,7 @@
       </c>
       <c r="C226" t="inlineStr">
         <is>
-          <t>Boy</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D226" t="inlineStr">
@@ -5246,7 +5250,7 @@
     </row>
     <row r="227">
       <c r="A227" t="n">
-        <v>206371</v>
+        <v>422371</v>
       </c>
       <c r="B227" t="inlineStr">
         <is>
@@ -5255,19 +5259,19 @@
       </c>
       <c r="C227" t="inlineStr">
         <is>
-          <t>Girl</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D227" t="inlineStr">
         <is>
-          <t>Isl</t>
+          <t>Msc</t>
         </is>
       </c>
       <c r="E227" t="inlineStr"/>
     </row>
     <row r="228">
       <c r="A228" t="n">
-        <v>915919</v>
+        <v>886375</v>
       </c>
       <c r="B228" t="inlineStr">
         <is>
@@ -5276,19 +5280,19 @@
       </c>
       <c r="C228" t="inlineStr">
         <is>
-          <t>Boy</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D228" t="inlineStr">
         <is>
-          <t>Isl</t>
+          <t>Msc</t>
         </is>
       </c>
       <c r="E228" t="inlineStr"/>
     </row>
     <row r="229">
       <c r="A229" t="n">
-        <v>190824</v>
+        <v>593135</v>
       </c>
       <c r="B229" t="inlineStr">
         <is>
@@ -5297,7 +5301,7 @@
       </c>
       <c r="C229" t="inlineStr">
         <is>
-          <t>Boy</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D229" t="inlineStr">
@@ -5309,7 +5313,7 @@
     </row>
     <row r="230">
       <c r="A230" t="n">
-        <v>856728</v>
+        <v>767757</v>
       </c>
       <c r="B230" t="inlineStr">
         <is>
@@ -5318,7 +5322,7 @@
       </c>
       <c r="C230" t="inlineStr">
         <is>
-          <t>Girl</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D230" t="inlineStr">
@@ -5326,15 +5330,11 @@
           <t>Msc</t>
         </is>
       </c>
-      <c r="E230" t="inlineStr">
-        <is>
-          <t>Naughty</t>
-        </is>
-      </c>
+      <c r="E230" t="inlineStr"/>
     </row>
     <row r="231">
       <c r="A231" t="n">
-        <v>986630</v>
+        <v>952080</v>
       </c>
       <c r="B231" t="inlineStr">
         <is>
@@ -5343,12 +5343,12 @@
       </c>
       <c r="C231" t="inlineStr">
         <is>
-          <t>Boy</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D231" t="inlineStr">
         <is>
-          <t>Msc</t>
+          <t>Isl</t>
         </is>
       </c>
       <c r="E231" t="inlineStr"/>

</xml_diff>

<commit_message>
Updated test excel sheet
</commit_message>
<xml_diff>
--- a/tests/students_test_data.xlsx
+++ b/tests/students_test_data.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E231"/>
+  <dimension ref="A1:E206"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -457,7 +457,7 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>556618</v>
+        <v>716273</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
@@ -471,14 +471,14 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Isl</t>
+          <t>Msc</t>
         </is>
       </c>
       <c r="E2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>439626</v>
+        <v>765285</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -495,11 +495,15 @@
           <t>Msc</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr"/>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Naughty</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>422078</v>
+        <v>997418</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -508,19 +512,23 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Male</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Msc</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr"/>
+          <t>Isl</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Naughty</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>231426</v>
+        <v>179864</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
@@ -537,15 +545,11 @@
           <t>Msc</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>Naughty</t>
-        </is>
-      </c>
+      <c r="E5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>768989</v>
+        <v>905458</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
@@ -554,7 +558,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Female</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -566,7 +570,7 @@
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>354126</v>
+        <v>885395</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
@@ -575,19 +579,19 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Female</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Isl</t>
+          <t>Msc</t>
         </is>
       </c>
       <c r="E7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>595140</v>
+        <v>688153</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
@@ -601,14 +605,14 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Msc</t>
+          <t>Isl</t>
         </is>
       </c>
       <c r="E8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>438894</v>
+        <v>161373</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
@@ -622,14 +626,14 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Msc</t>
+          <t>Isl</t>
         </is>
       </c>
       <c r="E9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>418319</v>
+        <v>613019</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
@@ -650,7 +654,7 @@
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>442768</v>
+        <v>747963</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
@@ -671,7 +675,7 @@
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>700245</v>
+        <v>366268</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
@@ -692,7 +696,7 @@
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>932445</v>
+        <v>533458</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
@@ -701,19 +705,19 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Female</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Msc</t>
+          <t>Isl</t>
         </is>
       </c>
       <c r="E13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>550953</v>
+        <v>675950</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
@@ -722,7 +726,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Female</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -734,7 +738,7 @@
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>703118</v>
+        <v>714177</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
@@ -743,7 +747,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Male</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -755,7 +759,7 @@
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>611011</v>
+        <v>651752</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
@@ -764,19 +768,23 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Male</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Isl</t>
-        </is>
-      </c>
-      <c r="E16" t="inlineStr"/>
+          <t>Msc</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Naughty</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>417040</v>
+        <v>599301</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
@@ -785,19 +793,19 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Male</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Isl</t>
+          <t>Msc</t>
         </is>
       </c>
       <c r="E17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>955101</v>
+        <v>983055</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
@@ -811,7 +819,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Msc</t>
+          <t>Isl</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -822,7 +830,7 @@
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>264831</v>
+        <v>168415</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
@@ -836,14 +844,14 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Isl</t>
+          <t>Msc</t>
         </is>
       </c>
       <c r="E19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>110494</v>
+        <v>606474</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
@@ -852,7 +860,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Female</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -860,15 +868,11 @@
           <t>Msc</t>
         </is>
       </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>Naughty</t>
-        </is>
-      </c>
+      <c r="E20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>756117</v>
+        <v>487594</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
@@ -882,14 +886,14 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Msc</t>
+          <t>Isl</t>
         </is>
       </c>
       <c r="E21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>368243</v>
+        <v>955193</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
@@ -898,7 +902,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Female</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -910,7 +914,7 @@
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>886449</v>
+        <v>470474</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
@@ -919,19 +923,19 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Male</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Isl</t>
+          <t>Msc</t>
         </is>
       </c>
       <c r="E23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>811978</v>
+        <v>940765</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
@@ -940,7 +944,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Female</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -948,11 +952,15 @@
           <t>Msc</t>
         </is>
       </c>
-      <c r="E24" t="inlineStr"/>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Naughty</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>719615</v>
+        <v>994882</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
@@ -966,14 +974,18 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Msc</t>
-        </is>
-      </c>
-      <c r="E25" t="inlineStr"/>
+          <t>Isl</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Naughty</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
-        <v>726064</v>
+        <v>753808</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
@@ -987,18 +999,14 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Msc</t>
-        </is>
-      </c>
-      <c r="E26" t="inlineStr">
-        <is>
-          <t>Weak in studies</t>
-        </is>
-      </c>
+          <t>Isl</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="n">
-        <v>770663</v>
+        <v>743704</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
@@ -1019,7 +1027,7 @@
     </row>
     <row r="28">
       <c r="A28" t="n">
-        <v>632975</v>
+        <v>919932</v>
       </c>
       <c r="B28" t="inlineStr">
         <is>
@@ -1033,14 +1041,14 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Msc</t>
+          <t>Isl</t>
         </is>
       </c>
       <c r="E28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="n">
-        <v>449232</v>
+        <v>819174</v>
       </c>
       <c r="B29" t="inlineStr">
         <is>
@@ -1054,14 +1062,14 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Isl</t>
+          <t>Msc</t>
         </is>
       </c>
       <c r="E29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="n">
-        <v>284090</v>
+        <v>174641</v>
       </c>
       <c r="B30" t="inlineStr">
         <is>
@@ -1082,7 +1090,7 @@
     </row>
     <row r="31">
       <c r="A31" t="n">
-        <v>981074</v>
+        <v>443827</v>
       </c>
       <c r="B31" t="inlineStr">
         <is>
@@ -1091,19 +1099,19 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Female</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Isl</t>
+          <t>Msc</t>
         </is>
       </c>
       <c r="E31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="n">
-        <v>400264</v>
+        <v>804012</v>
       </c>
       <c r="B32" t="inlineStr">
         <is>
@@ -1124,7 +1132,7 @@
     </row>
     <row r="33">
       <c r="A33" t="n">
-        <v>715586</v>
+        <v>852459</v>
       </c>
       <c r="B33" t="inlineStr">
         <is>
@@ -1133,19 +1141,19 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Female</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Msc</t>
+          <t>Isl</t>
         </is>
       </c>
       <c r="E33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="n">
-        <v>804889</v>
+        <v>842800</v>
       </c>
       <c r="B34" t="inlineStr">
         <is>
@@ -1154,7 +1162,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Female</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -1166,7 +1174,7 @@
     </row>
     <row r="35">
       <c r="A35" t="n">
-        <v>273518</v>
+        <v>292585</v>
       </c>
       <c r="B35" t="inlineStr">
         <is>
@@ -1175,19 +1183,19 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Male</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Isl</t>
+          <t>Msc</t>
         </is>
       </c>
       <c r="E35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="n">
-        <v>127017</v>
+        <v>670348</v>
       </c>
       <c r="B36" t="inlineStr">
         <is>
@@ -1196,19 +1204,19 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Female</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Msc</t>
+          <t>Isl</t>
         </is>
       </c>
       <c r="E36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="n">
-        <v>714244</v>
+        <v>468230</v>
       </c>
       <c r="B37" t="inlineStr">
         <is>
@@ -1222,18 +1230,14 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Isl</t>
-        </is>
-      </c>
-      <c r="E37" t="inlineStr">
-        <is>
-          <t>Naughty</t>
-        </is>
-      </c>
+          <t>Msc</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="n">
-        <v>710275</v>
+        <v>190596</v>
       </c>
       <c r="B38" t="inlineStr">
         <is>
@@ -1254,7 +1258,7 @@
     </row>
     <row r="39">
       <c r="A39" t="n">
-        <v>557873</v>
+        <v>665515</v>
       </c>
       <c r="B39" t="inlineStr">
         <is>
@@ -1275,7 +1279,7 @@
     </row>
     <row r="40">
       <c r="A40" t="n">
-        <v>325311</v>
+        <v>946594</v>
       </c>
       <c r="B40" t="inlineStr">
         <is>
@@ -1284,7 +1288,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Female</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -1296,7 +1300,7 @@
     </row>
     <row r="41">
       <c r="A41" t="n">
-        <v>884755</v>
+        <v>599106</v>
       </c>
       <c r="B41" t="inlineStr">
         <is>
@@ -1317,7 +1321,7 @@
     </row>
     <row r="42">
       <c r="A42" t="n">
-        <v>808404</v>
+        <v>347652</v>
       </c>
       <c r="B42" t="inlineStr">
         <is>
@@ -1326,7 +1330,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Female</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -1334,11 +1338,15 @@
           <t>Isl</t>
         </is>
       </c>
-      <c r="E42" t="inlineStr"/>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>Weak in studies</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="n">
-        <v>581753</v>
+        <v>351663</v>
       </c>
       <c r="B43" t="inlineStr">
         <is>
@@ -1347,7 +1355,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Female</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -1359,7 +1367,7 @@
     </row>
     <row r="44">
       <c r="A44" t="n">
-        <v>592647</v>
+        <v>897370</v>
       </c>
       <c r="B44" t="inlineStr">
         <is>
@@ -1373,14 +1381,14 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Msc</t>
+          <t>Isl</t>
         </is>
       </c>
       <c r="E44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="n">
-        <v>762029</v>
+        <v>302565</v>
       </c>
       <c r="B45" t="inlineStr">
         <is>
@@ -1394,14 +1402,14 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Msc</t>
+          <t>Isl</t>
         </is>
       </c>
       <c r="E45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="n">
-        <v>585750</v>
+        <v>748628</v>
       </c>
       <c r="B46" t="inlineStr">
         <is>
@@ -1410,19 +1418,19 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Female</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Isl</t>
+          <t>Msc</t>
         </is>
       </c>
       <c r="E46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="n">
-        <v>787167</v>
+        <v>763237</v>
       </c>
       <c r="B47" t="inlineStr">
         <is>
@@ -1431,19 +1439,19 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Female</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Msc</t>
+          <t>Isl</t>
         </is>
       </c>
       <c r="E47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="n">
-        <v>753554</v>
+        <v>966345</v>
       </c>
       <c r="B48" t="inlineStr">
         <is>
@@ -1452,7 +1460,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Male</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -1464,7 +1472,7 @@
     </row>
     <row r="49">
       <c r="A49" t="n">
-        <v>846376</v>
+        <v>451735</v>
       </c>
       <c r="B49" t="inlineStr">
         <is>
@@ -1485,7 +1493,7 @@
     </row>
     <row r="50">
       <c r="A50" t="n">
-        <v>881175</v>
+        <v>147347</v>
       </c>
       <c r="B50" t="inlineStr">
         <is>
@@ -1506,7 +1514,7 @@
     </row>
     <row r="51">
       <c r="A51" t="n">
-        <v>135481</v>
+        <v>387008</v>
       </c>
       <c r="B51" t="inlineStr">
         <is>
@@ -1515,7 +1523,7 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Female</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
@@ -1527,7 +1535,7 @@
     </row>
     <row r="52">
       <c r="A52" t="n">
-        <v>431046</v>
+        <v>712721</v>
       </c>
       <c r="B52" t="inlineStr">
         <is>
@@ -1536,7 +1544,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Male</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
@@ -1548,7 +1556,7 @@
     </row>
     <row r="53">
       <c r="A53" t="n">
-        <v>600855</v>
+        <v>807861</v>
       </c>
       <c r="B53" t="inlineStr">
         <is>
@@ -1565,15 +1573,11 @@
           <t>Msc</t>
         </is>
       </c>
-      <c r="E53" t="inlineStr">
-        <is>
-          <t>Naughty</t>
-        </is>
-      </c>
+      <c r="E53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="n">
-        <v>266048</v>
+        <v>284603</v>
       </c>
       <c r="B54" t="inlineStr">
         <is>
@@ -1582,19 +1586,19 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Male</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Isl</t>
+          <t>Msc</t>
         </is>
       </c>
       <c r="E54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="n">
-        <v>398424</v>
+        <v>963070</v>
       </c>
       <c r="B55" t="inlineStr">
         <is>
@@ -1615,7 +1619,7 @@
     </row>
     <row r="56">
       <c r="A56" t="n">
-        <v>844393</v>
+        <v>287483</v>
       </c>
       <c r="B56" t="inlineStr">
         <is>
@@ -1629,18 +1633,14 @@
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Isl</t>
-        </is>
-      </c>
-      <c r="E56" t="inlineStr">
-        <is>
-          <t>Naughty</t>
-        </is>
-      </c>
+          <t>Msc</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="n">
-        <v>254552</v>
+        <v>294348</v>
       </c>
       <c r="B57" t="inlineStr">
         <is>
@@ -1654,18 +1654,14 @@
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Isl</t>
-        </is>
-      </c>
-      <c r="E57" t="inlineStr">
-        <is>
-          <t>Naughty</t>
-        </is>
-      </c>
+          <t>Msc</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="n">
-        <v>829601</v>
+        <v>201581</v>
       </c>
       <c r="B58" t="inlineStr">
         <is>
@@ -1674,19 +1670,19 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Male</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Msc</t>
+          <t>Isl</t>
         </is>
       </c>
       <c r="E58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="n">
-        <v>393039</v>
+        <v>396830</v>
       </c>
       <c r="B59" t="inlineStr">
         <is>
@@ -1707,7 +1703,7 @@
     </row>
     <row r="60">
       <c r="A60" t="n">
-        <v>822193</v>
+        <v>115484</v>
       </c>
       <c r="B60" t="inlineStr">
         <is>
@@ -1716,7 +1712,7 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Female</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
@@ -1724,11 +1720,15 @@
           <t>Msc</t>
         </is>
       </c>
-      <c r="E60" t="inlineStr"/>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>Weak in studies</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="n">
-        <v>303037</v>
+        <v>714982</v>
       </c>
       <c r="B61" t="inlineStr">
         <is>
@@ -1749,7 +1749,7 @@
     </row>
     <row r="62">
       <c r="A62" t="n">
-        <v>101919</v>
+        <v>681645</v>
       </c>
       <c r="B62" t="inlineStr">
         <is>
@@ -1770,7 +1770,7 @@
     </row>
     <row r="63">
       <c r="A63" t="n">
-        <v>848723</v>
+        <v>538199</v>
       </c>
       <c r="B63" t="inlineStr">
         <is>
@@ -1779,19 +1779,19 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Female</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Isl</t>
+          <t>Msc</t>
         </is>
       </c>
       <c r="E63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="n">
-        <v>858106</v>
+        <v>913833</v>
       </c>
       <c r="B64" t="inlineStr">
         <is>
@@ -1800,19 +1800,19 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Male</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Isl</t>
+          <t>Msc</t>
         </is>
       </c>
       <c r="E64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="n">
-        <v>261958</v>
+        <v>163592</v>
       </c>
       <c r="B65" t="inlineStr">
         <is>
@@ -1833,7 +1833,7 @@
     </row>
     <row r="66">
       <c r="A66" t="n">
-        <v>650696</v>
+        <v>680944</v>
       </c>
       <c r="B66" t="inlineStr">
         <is>
@@ -1842,7 +1842,7 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Male</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
@@ -1854,7 +1854,7 @@
     </row>
     <row r="67">
       <c r="A67" t="n">
-        <v>457202</v>
+        <v>714012</v>
       </c>
       <c r="B67" t="inlineStr">
         <is>
@@ -1863,7 +1863,7 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Male</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
@@ -1875,7 +1875,7 @@
     </row>
     <row r="68">
       <c r="A68" t="n">
-        <v>942057</v>
+        <v>728574</v>
       </c>
       <c r="B68" t="inlineStr">
         <is>
@@ -1896,7 +1896,7 @@
     </row>
     <row r="69">
       <c r="A69" t="n">
-        <v>422836</v>
+        <v>401342</v>
       </c>
       <c r="B69" t="inlineStr">
         <is>
@@ -1905,19 +1905,23 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Female</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Isl</t>
-        </is>
-      </c>
-      <c r="E69" t="inlineStr"/>
+          <t>Msc</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>Naughty</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="n">
-        <v>411384</v>
+        <v>753246</v>
       </c>
       <c r="B70" t="inlineStr">
         <is>
@@ -1926,7 +1930,7 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Female</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
@@ -1938,7 +1942,7 @@
     </row>
     <row r="71">
       <c r="A71" t="n">
-        <v>266809</v>
+        <v>433840</v>
       </c>
       <c r="B71" t="inlineStr">
         <is>
@@ -1952,14 +1956,18 @@
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Msc</t>
-        </is>
-      </c>
-      <c r="E71" t="inlineStr"/>
+          <t>Isl</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>Weak in studies</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="n">
-        <v>917729</v>
+        <v>619071</v>
       </c>
       <c r="B72" t="inlineStr">
         <is>
@@ -1968,7 +1976,7 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Male</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
@@ -1980,7 +1988,7 @@
     </row>
     <row r="73">
       <c r="A73" t="n">
-        <v>544498</v>
+        <v>238747</v>
       </c>
       <c r="B73" t="inlineStr">
         <is>
@@ -1989,7 +1997,7 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>Female</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
@@ -2001,7 +2009,7 @@
     </row>
     <row r="74">
       <c r="A74" t="n">
-        <v>156946</v>
+        <v>252215</v>
       </c>
       <c r="B74" t="inlineStr">
         <is>
@@ -2010,7 +2018,7 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>Female</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
@@ -2022,7 +2030,7 @@
     </row>
     <row r="75">
       <c r="A75" t="n">
-        <v>748911</v>
+        <v>620141</v>
       </c>
       <c r="B75" t="inlineStr">
         <is>
@@ -2031,19 +2039,19 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>Male</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>Isl</t>
+          <t>Msc</t>
         </is>
       </c>
       <c r="E75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" t="n">
-        <v>652667</v>
+        <v>329791</v>
       </c>
       <c r="B76" t="inlineStr">
         <is>
@@ -2052,7 +2060,7 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Male</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
@@ -2064,7 +2072,7 @@
     </row>
     <row r="77">
       <c r="A77" t="n">
-        <v>889382</v>
+        <v>431037</v>
       </c>
       <c r="B77" t="inlineStr">
         <is>
@@ -2073,7 +2081,7 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Female</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
@@ -2085,7 +2093,7 @@
     </row>
     <row r="78">
       <c r="A78" t="n">
-        <v>994332</v>
+        <v>367705</v>
       </c>
       <c r="B78" t="inlineStr">
         <is>
@@ -2094,7 +2102,7 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>Male</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
@@ -2106,7 +2114,7 @@
     </row>
     <row r="79">
       <c r="A79" t="n">
-        <v>519893</v>
+        <v>789790</v>
       </c>
       <c r="B79" t="inlineStr">
         <is>
@@ -2127,7 +2135,7 @@
     </row>
     <row r="80">
       <c r="A80" t="n">
-        <v>105647</v>
+        <v>841271</v>
       </c>
       <c r="B80" t="inlineStr">
         <is>
@@ -2141,14 +2149,14 @@
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>Msc</t>
+          <t>Isl</t>
         </is>
       </c>
       <c r="E80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" t="n">
-        <v>877190</v>
+        <v>645664</v>
       </c>
       <c r="B81" t="inlineStr">
         <is>
@@ -2169,7 +2177,7 @@
     </row>
     <row r="82">
       <c r="A82" t="n">
-        <v>700858</v>
+        <v>605464</v>
       </c>
       <c r="B82" t="inlineStr">
         <is>
@@ -2183,14 +2191,14 @@
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>Msc</t>
+          <t>Isl</t>
         </is>
       </c>
       <c r="E82" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" t="n">
-        <v>491524</v>
+        <v>578746</v>
       </c>
       <c r="B83" t="inlineStr">
         <is>
@@ -2211,7 +2219,7 @@
     </row>
     <row r="84">
       <c r="A84" t="n">
-        <v>313081</v>
+        <v>329155</v>
       </c>
       <c r="B84" t="inlineStr">
         <is>
@@ -2225,14 +2233,14 @@
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>Isl</t>
+          <t>Msc</t>
         </is>
       </c>
       <c r="E84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" t="n">
-        <v>713280</v>
+        <v>833522</v>
       </c>
       <c r="B85" t="inlineStr">
         <is>
@@ -2246,14 +2254,14 @@
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>Msc</t>
+          <t>Isl</t>
         </is>
       </c>
       <c r="E85" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" t="n">
-        <v>522822</v>
+        <v>666379</v>
       </c>
       <c r="B86" t="inlineStr">
         <is>
@@ -2262,7 +2270,7 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>Female</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
@@ -2270,15 +2278,11 @@
           <t>Msc</t>
         </is>
       </c>
-      <c r="E86" t="inlineStr">
-        <is>
-          <t>Naughty</t>
-        </is>
-      </c>
+      <c r="E86" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" t="n">
-        <v>451111</v>
+        <v>314702</v>
       </c>
       <c r="B87" t="inlineStr">
         <is>
@@ -2287,19 +2291,19 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>Female</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>Isl</t>
+          <t>Msc</t>
         </is>
       </c>
       <c r="E87" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" t="n">
-        <v>276364</v>
+        <v>620699</v>
       </c>
       <c r="B88" t="inlineStr">
         <is>
@@ -2313,14 +2317,14 @@
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>Msc</t>
+          <t>Isl</t>
         </is>
       </c>
       <c r="E88" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" t="n">
-        <v>499376</v>
+        <v>412251</v>
       </c>
       <c r="B89" t="inlineStr">
         <is>
@@ -2334,14 +2338,14 @@
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>Msc</t>
+          <t>Isl</t>
         </is>
       </c>
       <c r="E89" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" t="n">
-        <v>429189</v>
+        <v>438712</v>
       </c>
       <c r="B90" t="inlineStr">
         <is>
@@ -2350,19 +2354,19 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>Male</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>Isl</t>
+          <t>Msc</t>
         </is>
       </c>
       <c r="E90" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" t="n">
-        <v>221871</v>
+        <v>381143</v>
       </c>
       <c r="B91" t="inlineStr">
         <is>
@@ -2371,19 +2375,19 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>Female</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>Isl</t>
+          <t>Msc</t>
         </is>
       </c>
       <c r="E91" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" t="n">
-        <v>932342</v>
+        <v>723107</v>
       </c>
       <c r="B92" t="inlineStr">
         <is>
@@ -2404,7 +2408,7 @@
     </row>
     <row r="93">
       <c r="A93" t="n">
-        <v>747095</v>
+        <v>567312</v>
       </c>
       <c r="B93" t="inlineStr">
         <is>
@@ -2413,7 +2417,7 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>Male</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
@@ -2421,11 +2425,15 @@
           <t>Msc</t>
         </is>
       </c>
-      <c r="E93" t="inlineStr"/>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>Naughty</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="n">
-        <v>673359</v>
+        <v>301467</v>
       </c>
       <c r="B94" t="inlineStr">
         <is>
@@ -2439,18 +2447,14 @@
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>Isl</t>
-        </is>
-      </c>
-      <c r="E94" t="inlineStr">
-        <is>
-          <t>Weak in studies</t>
-        </is>
-      </c>
+          <t>Msc</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" t="n">
-        <v>671800</v>
+        <v>658173</v>
       </c>
       <c r="B95" t="inlineStr">
         <is>
@@ -2471,7 +2475,7 @@
     </row>
     <row r="96">
       <c r="A96" t="n">
-        <v>105327</v>
+        <v>137102</v>
       </c>
       <c r="B96" t="inlineStr">
         <is>
@@ -2480,19 +2484,19 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>Female</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>Isl</t>
+          <t>Msc</t>
         </is>
       </c>
       <c r="E96" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" t="n">
-        <v>146561</v>
+        <v>559079</v>
       </c>
       <c r="B97" t="inlineStr">
         <is>
@@ -2506,14 +2510,18 @@
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>Isl</t>
-        </is>
-      </c>
-      <c r="E97" t="inlineStr"/>
+          <t>Msc</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>Naughty</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="n">
-        <v>210728</v>
+        <v>139995</v>
       </c>
       <c r="B98" t="inlineStr">
         <is>
@@ -2522,7 +2530,7 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>Female</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
@@ -2534,7 +2542,7 @@
     </row>
     <row r="99">
       <c r="A99" t="n">
-        <v>405592</v>
+        <v>296480</v>
       </c>
       <c r="B99" t="inlineStr">
         <is>
@@ -2543,19 +2551,19 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>Female</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>Isl</t>
+          <t>Msc</t>
         </is>
       </c>
       <c r="E99" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" t="n">
-        <v>631716</v>
+        <v>353364</v>
       </c>
       <c r="B100" t="inlineStr">
         <is>
@@ -2564,7 +2572,7 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>Male</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
@@ -2576,7 +2584,7 @@
     </row>
     <row r="101">
       <c r="A101" t="n">
-        <v>958502</v>
+        <v>835444</v>
       </c>
       <c r="B101" t="inlineStr">
         <is>
@@ -2597,7 +2605,7 @@
     </row>
     <row r="102">
       <c r="A102" t="n">
-        <v>770007</v>
+        <v>864618</v>
       </c>
       <c r="B102" t="inlineStr">
         <is>
@@ -2611,14 +2619,14 @@
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>Isl</t>
+          <t>Msc</t>
         </is>
       </c>
       <c r="E102" t="inlineStr"/>
     </row>
     <row r="103">
       <c r="A103" t="n">
-        <v>816671</v>
+        <v>105326</v>
       </c>
       <c r="B103" t="inlineStr">
         <is>
@@ -2627,7 +2635,7 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>Female</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
@@ -2639,7 +2647,7 @@
     </row>
     <row r="104">
       <c r="A104" t="n">
-        <v>858020</v>
+        <v>494075</v>
       </c>
       <c r="B104" t="inlineStr">
         <is>
@@ -2648,19 +2656,19 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>Female</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>Msc</t>
+          <t>Isl</t>
         </is>
       </c>
       <c r="E104" t="inlineStr"/>
     </row>
     <row r="105">
       <c r="A105" t="n">
-        <v>100808</v>
+        <v>979392</v>
       </c>
       <c r="B105" t="inlineStr">
         <is>
@@ -2669,7 +2677,7 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>Female</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
@@ -2681,7 +2689,7 @@
     </row>
     <row r="106">
       <c r="A106" t="n">
-        <v>947317</v>
+        <v>334539</v>
       </c>
       <c r="B106" t="inlineStr">
         <is>
@@ -2690,19 +2698,19 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>Female</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>Isl</t>
+          <t>Msc</t>
         </is>
       </c>
       <c r="E106" t="inlineStr"/>
     </row>
     <row r="107">
       <c r="A107" t="n">
-        <v>478843</v>
+        <v>339342</v>
       </c>
       <c r="B107" t="inlineStr">
         <is>
@@ -2716,18 +2724,14 @@
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>Isl</t>
-        </is>
-      </c>
-      <c r="E107" t="inlineStr">
-        <is>
-          <t>Naughty</t>
-        </is>
-      </c>
+          <t>Msc</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr"/>
     </row>
     <row r="108">
       <c r="A108" t="n">
-        <v>869557</v>
+        <v>142771</v>
       </c>
       <c r="B108" t="inlineStr">
         <is>
@@ -2741,14 +2745,14 @@
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>Isl</t>
+          <t>Msc</t>
         </is>
       </c>
       <c r="E108" t="inlineStr"/>
     </row>
     <row r="109">
       <c r="A109" t="n">
-        <v>834849</v>
+        <v>104040</v>
       </c>
       <c r="B109" t="inlineStr">
         <is>
@@ -2757,7 +2761,7 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>Male</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
@@ -2769,7 +2773,7 @@
     </row>
     <row r="110">
       <c r="A110" t="n">
-        <v>794334</v>
+        <v>186578</v>
       </c>
       <c r="B110" t="inlineStr">
         <is>
@@ -2778,7 +2782,7 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>Female</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
@@ -2786,11 +2790,15 @@
           <t>Isl</t>
         </is>
       </c>
-      <c r="E110" t="inlineStr"/>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>Naughty</t>
+        </is>
+      </c>
     </row>
     <row r="111">
       <c r="A111" t="n">
-        <v>638525</v>
+        <v>494765</v>
       </c>
       <c r="B111" t="inlineStr">
         <is>
@@ -2811,7 +2819,7 @@
     </row>
     <row r="112">
       <c r="A112" t="n">
-        <v>853067</v>
+        <v>431644</v>
       </c>
       <c r="B112" t="inlineStr">
         <is>
@@ -2828,11 +2836,15 @@
           <t>Msc</t>
         </is>
       </c>
-      <c r="E112" t="inlineStr"/>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>Naughty</t>
+        </is>
+      </c>
     </row>
     <row r="113">
       <c r="A113" t="n">
-        <v>103329</v>
+        <v>281939</v>
       </c>
       <c r="B113" t="inlineStr">
         <is>
@@ -2853,7 +2865,7 @@
     </row>
     <row r="114">
       <c r="A114" t="n">
-        <v>665955</v>
+        <v>783598</v>
       </c>
       <c r="B114" t="inlineStr">
         <is>
@@ -2867,14 +2879,14 @@
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>Isl</t>
+          <t>Msc</t>
         </is>
       </c>
       <c r="E114" t="inlineStr"/>
     </row>
     <row r="115">
       <c r="A115" t="n">
-        <v>288585</v>
+        <v>229899</v>
       </c>
       <c r="B115" t="inlineStr">
         <is>
@@ -2895,7 +2907,7 @@
     </row>
     <row r="116">
       <c r="A116" t="n">
-        <v>349296</v>
+        <v>777045</v>
       </c>
       <c r="B116" t="inlineStr">
         <is>
@@ -2904,19 +2916,19 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>Female</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>Msc</t>
+          <t>Isl</t>
         </is>
       </c>
       <c r="E116" t="inlineStr"/>
     </row>
     <row r="117">
       <c r="A117" t="n">
-        <v>868351</v>
+        <v>818347</v>
       </c>
       <c r="B117" t="inlineStr">
         <is>
@@ -2925,7 +2937,7 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>Female</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
@@ -2937,7 +2949,7 @@
     </row>
     <row r="118">
       <c r="A118" t="n">
-        <v>290870</v>
+        <v>925536</v>
       </c>
       <c r="B118" t="inlineStr">
         <is>
@@ -2946,19 +2958,19 @@
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>Male</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>Isl</t>
+          <t>Msc</t>
         </is>
       </c>
       <c r="E118" t="inlineStr"/>
     </row>
     <row r="119">
       <c r="A119" t="n">
-        <v>242230</v>
+        <v>101213</v>
       </c>
       <c r="B119" t="inlineStr">
         <is>
@@ -2967,19 +2979,19 @@
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>Female</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>Msc</t>
+          <t>Isl</t>
         </is>
       </c>
       <c r="E119" t="inlineStr"/>
     </row>
     <row r="120">
       <c r="A120" t="n">
-        <v>241888</v>
+        <v>100319</v>
       </c>
       <c r="B120" t="inlineStr">
         <is>
@@ -3000,7 +3012,7 @@
     </row>
     <row r="121">
       <c r="A121" t="n">
-        <v>983334</v>
+        <v>913778</v>
       </c>
       <c r="B121" t="inlineStr">
         <is>
@@ -3021,7 +3033,7 @@
     </row>
     <row r="122">
       <c r="A122" t="n">
-        <v>551203</v>
+        <v>735936</v>
       </c>
       <c r="B122" t="inlineStr">
         <is>
@@ -3042,7 +3054,7 @@
     </row>
     <row r="123">
       <c r="A123" t="n">
-        <v>644775</v>
+        <v>267830</v>
       </c>
       <c r="B123" t="inlineStr">
         <is>
@@ -3051,19 +3063,19 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>Male</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>Isl</t>
+          <t>Msc</t>
         </is>
       </c>
       <c r="E123" t="inlineStr"/>
     </row>
     <row r="124">
       <c r="A124" t="n">
-        <v>915267</v>
+        <v>603603</v>
       </c>
       <c r="B124" t="inlineStr">
         <is>
@@ -3077,14 +3089,14 @@
       </c>
       <c r="D124" t="inlineStr">
         <is>
-          <t>Isl</t>
+          <t>Msc</t>
         </is>
       </c>
       <c r="E124" t="inlineStr"/>
     </row>
     <row r="125">
       <c r="A125" t="n">
-        <v>947104</v>
+        <v>184482</v>
       </c>
       <c r="B125" t="inlineStr">
         <is>
@@ -3093,7 +3105,7 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>Male</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D125" t="inlineStr">
@@ -3105,7 +3117,7 @@
     </row>
     <row r="126">
       <c r="A126" t="n">
-        <v>179281</v>
+        <v>753468</v>
       </c>
       <c r="B126" t="inlineStr">
         <is>
@@ -3114,19 +3126,19 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>Male</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D126" t="inlineStr">
         <is>
-          <t>Msc</t>
+          <t>Isl</t>
         </is>
       </c>
       <c r="E126" t="inlineStr"/>
     </row>
     <row r="127">
       <c r="A127" t="n">
-        <v>136397</v>
+        <v>422944</v>
       </c>
       <c r="B127" t="inlineStr">
         <is>
@@ -3140,14 +3152,18 @@
       </c>
       <c r="D127" t="inlineStr">
         <is>
-          <t>Isl</t>
-        </is>
-      </c>
-      <c r="E127" t="inlineStr"/>
+          <t>Msc</t>
+        </is>
+      </c>
+      <c r="E127" t="inlineStr">
+        <is>
+          <t>Weak in studies</t>
+        </is>
+      </c>
     </row>
     <row r="128">
       <c r="A128" t="n">
-        <v>911209</v>
+        <v>347279</v>
       </c>
       <c r="B128" t="inlineStr">
         <is>
@@ -3168,7 +3184,7 @@
     </row>
     <row r="129">
       <c r="A129" t="n">
-        <v>794049</v>
+        <v>869248</v>
       </c>
       <c r="B129" t="inlineStr">
         <is>
@@ -3177,7 +3193,7 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>Male</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D129" t="inlineStr">
@@ -3189,7 +3205,7 @@
     </row>
     <row r="130">
       <c r="A130" t="n">
-        <v>795496</v>
+        <v>262359</v>
       </c>
       <c r="B130" t="inlineStr">
         <is>
@@ -3198,7 +3214,7 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>Female</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D130" t="inlineStr">
@@ -3206,15 +3222,11 @@
           <t>Msc</t>
         </is>
       </c>
-      <c r="E130" t="inlineStr">
-        <is>
-          <t>Weak in studies</t>
-        </is>
-      </c>
+      <c r="E130" t="inlineStr"/>
     </row>
     <row r="131">
       <c r="A131" t="n">
-        <v>305910</v>
+        <v>894822</v>
       </c>
       <c r="B131" t="inlineStr">
         <is>
@@ -3235,7 +3247,7 @@
     </row>
     <row r="132">
       <c r="A132" t="n">
-        <v>210230</v>
+        <v>484121</v>
       </c>
       <c r="B132" t="inlineStr">
         <is>
@@ -3244,19 +3256,19 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>Male</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D132" t="inlineStr">
         <is>
-          <t>Msc</t>
+          <t>Isl</t>
         </is>
       </c>
       <c r="E132" t="inlineStr"/>
     </row>
     <row r="133">
       <c r="A133" t="n">
-        <v>334791</v>
+        <v>418791</v>
       </c>
       <c r="B133" t="inlineStr">
         <is>
@@ -3265,23 +3277,19 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>Male</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D133" t="inlineStr">
         <is>
-          <t>Isl</t>
-        </is>
-      </c>
-      <c r="E133" t="inlineStr">
-        <is>
-          <t>Naughty</t>
-        </is>
-      </c>
+          <t>Msc</t>
+        </is>
+      </c>
+      <c r="E133" t="inlineStr"/>
     </row>
     <row r="134">
       <c r="A134" t="n">
-        <v>124149</v>
+        <v>197831</v>
       </c>
       <c r="B134" t="inlineStr">
         <is>
@@ -3302,7 +3310,7 @@
     </row>
     <row r="135">
       <c r="A135" t="n">
-        <v>432811</v>
+        <v>793298</v>
       </c>
       <c r="B135" t="inlineStr">
         <is>
@@ -3323,7 +3331,7 @@
     </row>
     <row r="136">
       <c r="A136" t="n">
-        <v>636816</v>
+        <v>777989</v>
       </c>
       <c r="B136" t="inlineStr">
         <is>
@@ -3337,14 +3345,14 @@
       </c>
       <c r="D136" t="inlineStr">
         <is>
-          <t>Msc</t>
+          <t>Isl</t>
         </is>
       </c>
       <c r="E136" t="inlineStr"/>
     </row>
     <row r="137">
       <c r="A137" t="n">
-        <v>990284</v>
+        <v>277641</v>
       </c>
       <c r="B137" t="inlineStr">
         <is>
@@ -3365,7 +3373,7 @@
     </row>
     <row r="138">
       <c r="A138" t="n">
-        <v>516400</v>
+        <v>178296</v>
       </c>
       <c r="B138" t="inlineStr">
         <is>
@@ -3374,19 +3382,19 @@
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>Male</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D138" t="inlineStr">
         <is>
-          <t>Isl</t>
+          <t>Msc</t>
         </is>
       </c>
       <c r="E138" t="inlineStr"/>
     </row>
     <row r="139">
       <c r="A139" t="n">
-        <v>778043</v>
+        <v>212274</v>
       </c>
       <c r="B139" t="inlineStr">
         <is>
@@ -3400,14 +3408,14 @@
       </c>
       <c r="D139" t="inlineStr">
         <is>
-          <t>Isl</t>
+          <t>Msc</t>
         </is>
       </c>
       <c r="E139" t="inlineStr"/>
     </row>
     <row r="140">
       <c r="A140" t="n">
-        <v>204471</v>
+        <v>597670</v>
       </c>
       <c r="B140" t="inlineStr">
         <is>
@@ -3428,7 +3436,7 @@
     </row>
     <row r="141">
       <c r="A141" t="n">
-        <v>179109</v>
+        <v>977401</v>
       </c>
       <c r="B141" t="inlineStr">
         <is>
@@ -3449,7 +3457,7 @@
     </row>
     <row r="142">
       <c r="A142" t="n">
-        <v>776595</v>
+        <v>826301</v>
       </c>
       <c r="B142" t="inlineStr">
         <is>
@@ -3470,7 +3478,7 @@
     </row>
     <row r="143">
       <c r="A143" t="n">
-        <v>281942</v>
+        <v>216107</v>
       </c>
       <c r="B143" t="inlineStr">
         <is>
@@ -3491,7 +3499,7 @@
     </row>
     <row r="144">
       <c r="A144" t="n">
-        <v>530758</v>
+        <v>765454</v>
       </c>
       <c r="B144" t="inlineStr">
         <is>
@@ -3500,7 +3508,7 @@
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>Male</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D144" t="inlineStr">
@@ -3512,7 +3520,7 @@
     </row>
     <row r="145">
       <c r="A145" t="n">
-        <v>827035</v>
+        <v>782448</v>
       </c>
       <c r="B145" t="inlineStr">
         <is>
@@ -3521,7 +3529,7 @@
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>Male</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D145" t="inlineStr">
@@ -3533,7 +3541,7 @@
     </row>
     <row r="146">
       <c r="A146" t="n">
-        <v>226372</v>
+        <v>705974</v>
       </c>
       <c r="B146" t="inlineStr">
         <is>
@@ -3542,7 +3550,7 @@
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>Female</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D146" t="inlineStr">
@@ -3554,7 +3562,7 @@
     </row>
     <row r="147">
       <c r="A147" t="n">
-        <v>995976</v>
+        <v>715673</v>
       </c>
       <c r="B147" t="inlineStr">
         <is>
@@ -3563,19 +3571,19 @@
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>Male</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D147" t="inlineStr">
         <is>
-          <t>Isl</t>
+          <t>Msc</t>
         </is>
       </c>
       <c r="E147" t="inlineStr"/>
     </row>
     <row r="148">
       <c r="A148" t="n">
-        <v>990771</v>
+        <v>468485</v>
       </c>
       <c r="B148" t="inlineStr">
         <is>
@@ -3589,14 +3597,14 @@
       </c>
       <c r="D148" t="inlineStr">
         <is>
-          <t>Msc</t>
+          <t>Isl</t>
         </is>
       </c>
       <c r="E148" t="inlineStr"/>
     </row>
     <row r="149">
       <c r="A149" t="n">
-        <v>640630</v>
+        <v>277919</v>
       </c>
       <c r="B149" t="inlineStr">
         <is>
@@ -3610,14 +3618,18 @@
       </c>
       <c r="D149" t="inlineStr">
         <is>
-          <t>Msc</t>
-        </is>
-      </c>
-      <c r="E149" t="inlineStr"/>
+          <t>Isl</t>
+        </is>
+      </c>
+      <c r="E149" t="inlineStr">
+        <is>
+          <t>Naughty</t>
+        </is>
+      </c>
     </row>
     <row r="150">
       <c r="A150" t="n">
-        <v>623403</v>
+        <v>225366</v>
       </c>
       <c r="B150" t="inlineStr">
         <is>
@@ -3626,7 +3638,7 @@
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>Female</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D150" t="inlineStr">
@@ -3638,7 +3650,7 @@
     </row>
     <row r="151">
       <c r="A151" t="n">
-        <v>314203</v>
+        <v>904991</v>
       </c>
       <c r="B151" t="inlineStr">
         <is>
@@ -3659,7 +3671,7 @@
     </row>
     <row r="152">
       <c r="A152" t="n">
-        <v>114494</v>
+        <v>897005</v>
       </c>
       <c r="B152" t="inlineStr">
         <is>
@@ -3673,14 +3685,14 @@
       </c>
       <c r="D152" t="inlineStr">
         <is>
-          <t>Msc</t>
+          <t>Isl</t>
         </is>
       </c>
       <c r="E152" t="inlineStr"/>
     </row>
     <row r="153">
       <c r="A153" t="n">
-        <v>713088</v>
+        <v>798861</v>
       </c>
       <c r="B153" t="inlineStr">
         <is>
@@ -3689,7 +3701,7 @@
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>Male</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D153" t="inlineStr">
@@ -3701,7 +3713,7 @@
     </row>
     <row r="154">
       <c r="A154" t="n">
-        <v>836599</v>
+        <v>785240</v>
       </c>
       <c r="B154" t="inlineStr">
         <is>
@@ -3710,7 +3722,7 @@
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>Male</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D154" t="inlineStr">
@@ -3722,7 +3734,7 @@
     </row>
     <row r="155">
       <c r="A155" t="n">
-        <v>576946</v>
+        <v>467998</v>
       </c>
       <c r="B155" t="inlineStr">
         <is>
@@ -3731,7 +3743,7 @@
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>Female</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D155" t="inlineStr">
@@ -3743,7 +3755,7 @@
     </row>
     <row r="156">
       <c r="A156" t="n">
-        <v>199333</v>
+        <v>987420</v>
       </c>
       <c r="B156" t="inlineStr">
         <is>
@@ -3752,19 +3764,19 @@
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>Male</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D156" t="inlineStr">
         <is>
-          <t>Msc</t>
+          <t>Isl</t>
         </is>
       </c>
       <c r="E156" t="inlineStr"/>
     </row>
     <row r="157">
       <c r="A157" t="n">
-        <v>504651</v>
+        <v>127136</v>
       </c>
       <c r="B157" t="inlineStr">
         <is>
@@ -3773,19 +3785,19 @@
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>Female</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D157" t="inlineStr">
         <is>
-          <t>Msc</t>
+          <t>Isl</t>
         </is>
       </c>
       <c r="E157" t="inlineStr"/>
     </row>
     <row r="158">
       <c r="A158" t="n">
-        <v>245979</v>
+        <v>597532</v>
       </c>
       <c r="B158" t="inlineStr">
         <is>
@@ -3794,19 +3806,19 @@
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>Male</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D158" t="inlineStr">
         <is>
-          <t>Msc</t>
+          <t>Isl</t>
         </is>
       </c>
       <c r="E158" t="inlineStr"/>
     </row>
     <row r="159">
       <c r="A159" t="n">
-        <v>156038</v>
+        <v>111548</v>
       </c>
       <c r="B159" t="inlineStr">
         <is>
@@ -3820,14 +3832,14 @@
       </c>
       <c r="D159" t="inlineStr">
         <is>
-          <t>Msc</t>
+          <t>Isl</t>
         </is>
       </c>
       <c r="E159" t="inlineStr"/>
     </row>
     <row r="160">
       <c r="A160" t="n">
-        <v>207017</v>
+        <v>461538</v>
       </c>
       <c r="B160" t="inlineStr">
         <is>
@@ -3836,19 +3848,19 @@
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>Female</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D160" t="inlineStr">
         <is>
-          <t>Msc</t>
+          <t>Isl</t>
         </is>
       </c>
       <c r="E160" t="inlineStr"/>
     </row>
     <row r="161">
       <c r="A161" t="n">
-        <v>821697</v>
+        <v>159014</v>
       </c>
       <c r="B161" t="inlineStr">
         <is>
@@ -3869,7 +3881,7 @@
     </row>
     <row r="162">
       <c r="A162" t="n">
-        <v>380867</v>
+        <v>956182</v>
       </c>
       <c r="B162" t="inlineStr">
         <is>
@@ -3878,7 +3890,7 @@
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>Female</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D162" t="inlineStr">
@@ -3890,7 +3902,7 @@
     </row>
     <row r="163">
       <c r="A163" t="n">
-        <v>889998</v>
+        <v>882910</v>
       </c>
       <c r="B163" t="inlineStr">
         <is>
@@ -3899,19 +3911,19 @@
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>Male</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D163" t="inlineStr">
         <is>
-          <t>Isl</t>
+          <t>Msc</t>
         </is>
       </c>
       <c r="E163" t="inlineStr"/>
     </row>
     <row r="164">
       <c r="A164" t="n">
-        <v>769589</v>
+        <v>598845</v>
       </c>
       <c r="B164" t="inlineStr">
         <is>
@@ -3932,7 +3944,7 @@
     </row>
     <row r="165">
       <c r="A165" t="n">
-        <v>106884</v>
+        <v>346801</v>
       </c>
       <c r="B165" t="inlineStr">
         <is>
@@ -3946,14 +3958,14 @@
       </c>
       <c r="D165" t="inlineStr">
         <is>
-          <t>Isl</t>
+          <t>Msc</t>
         </is>
       </c>
       <c r="E165" t="inlineStr"/>
     </row>
     <row r="166">
       <c r="A166" t="n">
-        <v>197478</v>
+        <v>132864</v>
       </c>
       <c r="B166" t="inlineStr">
         <is>
@@ -3962,7 +3974,7 @@
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>Male</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D166" t="inlineStr">
@@ -3974,7 +3986,7 @@
     </row>
     <row r="167">
       <c r="A167" t="n">
-        <v>350329</v>
+        <v>734927</v>
       </c>
       <c r="B167" t="inlineStr">
         <is>
@@ -3995,7 +4007,7 @@
     </row>
     <row r="168">
       <c r="A168" t="n">
-        <v>270592</v>
+        <v>788412</v>
       </c>
       <c r="B168" t="inlineStr">
         <is>
@@ -4009,14 +4021,14 @@
       </c>
       <c r="D168" t="inlineStr">
         <is>
-          <t>Msc</t>
+          <t>Isl</t>
         </is>
       </c>
       <c r="E168" t="inlineStr"/>
     </row>
     <row r="169">
       <c r="A169" t="n">
-        <v>843959</v>
+        <v>700413</v>
       </c>
       <c r="B169" t="inlineStr">
         <is>
@@ -4037,7 +4049,7 @@
     </row>
     <row r="170">
       <c r="A170" t="n">
-        <v>622498</v>
+        <v>757613</v>
       </c>
       <c r="B170" t="inlineStr">
         <is>
@@ -4051,14 +4063,14 @@
       </c>
       <c r="D170" t="inlineStr">
         <is>
-          <t>Msc</t>
+          <t>Isl</t>
         </is>
       </c>
       <c r="E170" t="inlineStr"/>
     </row>
     <row r="171">
       <c r="A171" t="n">
-        <v>921465</v>
+        <v>646421</v>
       </c>
       <c r="B171" t="inlineStr">
         <is>
@@ -4079,7 +4091,7 @@
     </row>
     <row r="172">
       <c r="A172" t="n">
-        <v>782149</v>
+        <v>389280</v>
       </c>
       <c r="B172" t="inlineStr">
         <is>
@@ -4088,19 +4100,19 @@
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>Male</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D172" t="inlineStr">
         <is>
-          <t>Msc</t>
+          <t>Isl</t>
         </is>
       </c>
       <c r="E172" t="inlineStr"/>
     </row>
     <row r="173">
       <c r="A173" t="n">
-        <v>116890</v>
+        <v>860915</v>
       </c>
       <c r="B173" t="inlineStr">
         <is>
@@ -4114,14 +4126,14 @@
       </c>
       <c r="D173" t="inlineStr">
         <is>
-          <t>Msc</t>
+          <t>Isl</t>
         </is>
       </c>
       <c r="E173" t="inlineStr"/>
     </row>
     <row r="174">
       <c r="A174" t="n">
-        <v>192648</v>
+        <v>196600</v>
       </c>
       <c r="B174" t="inlineStr">
         <is>
@@ -4130,7 +4142,7 @@
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>Female</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D174" t="inlineStr">
@@ -4142,7 +4154,7 @@
     </row>
     <row r="175">
       <c r="A175" t="n">
-        <v>895720</v>
+        <v>385942</v>
       </c>
       <c r="B175" t="inlineStr">
         <is>
@@ -4156,14 +4168,14 @@
       </c>
       <c r="D175" t="inlineStr">
         <is>
-          <t>Isl</t>
+          <t>Msc</t>
         </is>
       </c>
       <c r="E175" t="inlineStr"/>
     </row>
     <row r="176">
       <c r="A176" t="n">
-        <v>654396</v>
+        <v>472091</v>
       </c>
       <c r="B176" t="inlineStr">
         <is>
@@ -4172,7 +4184,7 @@
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>Male</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D176" t="inlineStr">
@@ -4184,7 +4196,7 @@
     </row>
     <row r="177">
       <c r="A177" t="n">
-        <v>787226</v>
+        <v>797553</v>
       </c>
       <c r="B177" t="inlineStr">
         <is>
@@ -4193,7 +4205,7 @@
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>Female</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D177" t="inlineStr">
@@ -4205,7 +4217,7 @@
     </row>
     <row r="178">
       <c r="A178" t="n">
-        <v>318843</v>
+        <v>989529</v>
       </c>
       <c r="B178" t="inlineStr">
         <is>
@@ -4214,7 +4226,7 @@
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>Female</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D178" t="inlineStr">
@@ -4226,7 +4238,7 @@
     </row>
     <row r="179">
       <c r="A179" t="n">
-        <v>164101</v>
+        <v>233138</v>
       </c>
       <c r="B179" t="inlineStr">
         <is>
@@ -4247,7 +4259,7 @@
     </row>
     <row r="180">
       <c r="A180" t="n">
-        <v>988188</v>
+        <v>628000</v>
       </c>
       <c r="B180" t="inlineStr">
         <is>
@@ -4256,19 +4268,19 @@
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>Male</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D180" t="inlineStr">
         <is>
-          <t>Isl</t>
+          <t>Msc</t>
         </is>
       </c>
       <c r="E180" t="inlineStr"/>
     </row>
     <row r="181">
       <c r="A181" t="n">
-        <v>353272</v>
+        <v>856181</v>
       </c>
       <c r="B181" t="inlineStr">
         <is>
@@ -4289,7 +4301,7 @@
     </row>
     <row r="182">
       <c r="A182" t="n">
-        <v>611577</v>
+        <v>365256</v>
       </c>
       <c r="B182" t="inlineStr">
         <is>
@@ -4310,7 +4322,7 @@
     </row>
     <row r="183">
       <c r="A183" t="n">
-        <v>613486</v>
+        <v>106952</v>
       </c>
       <c r="B183" t="inlineStr">
         <is>
@@ -4324,14 +4336,14 @@
       </c>
       <c r="D183" t="inlineStr">
         <is>
-          <t>Msc</t>
+          <t>Isl</t>
         </is>
       </c>
       <c r="E183" t="inlineStr"/>
     </row>
     <row r="184">
       <c r="A184" t="n">
-        <v>113856</v>
+        <v>863920</v>
       </c>
       <c r="B184" t="inlineStr">
         <is>
@@ -4340,7 +4352,7 @@
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>Male</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D184" t="inlineStr">
@@ -4348,15 +4360,11 @@
           <t>Isl</t>
         </is>
       </c>
-      <c r="E184" t="inlineStr">
-        <is>
-          <t>Naughty</t>
-        </is>
-      </c>
+      <c r="E184" t="inlineStr"/>
     </row>
     <row r="185">
       <c r="A185" t="n">
-        <v>716906</v>
+        <v>265402</v>
       </c>
       <c r="B185" t="inlineStr">
         <is>
@@ -4370,14 +4378,14 @@
       </c>
       <c r="D185" t="inlineStr">
         <is>
-          <t>Isl</t>
+          <t>Msc</t>
         </is>
       </c>
       <c r="E185" t="inlineStr"/>
     </row>
     <row r="186">
       <c r="A186" t="n">
-        <v>486066</v>
+        <v>447796</v>
       </c>
       <c r="B186" t="inlineStr">
         <is>
@@ -4398,7 +4406,7 @@
     </row>
     <row r="187">
       <c r="A187" t="n">
-        <v>842790</v>
+        <v>277695</v>
       </c>
       <c r="B187" t="inlineStr">
         <is>
@@ -4407,19 +4415,19 @@
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>Female</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D187" t="inlineStr">
         <is>
-          <t>Msc</t>
+          <t>Isl</t>
         </is>
       </c>
       <c r="E187" t="inlineStr"/>
     </row>
     <row r="188">
       <c r="A188" t="n">
-        <v>844589</v>
+        <v>777771</v>
       </c>
       <c r="B188" t="inlineStr">
         <is>
@@ -4440,7 +4448,7 @@
     </row>
     <row r="189">
       <c r="A189" t="n">
-        <v>202062</v>
+        <v>694446</v>
       </c>
       <c r="B189" t="inlineStr">
         <is>
@@ -4449,23 +4457,19 @@
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>Male</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D189" t="inlineStr">
         <is>
-          <t>Isl</t>
-        </is>
-      </c>
-      <c r="E189" t="inlineStr">
-        <is>
-          <t>Weak in studies</t>
-        </is>
-      </c>
+          <t>Msc</t>
+        </is>
+      </c>
+      <c r="E189" t="inlineStr"/>
     </row>
     <row r="190">
       <c r="A190" t="n">
-        <v>791430</v>
+        <v>486531</v>
       </c>
       <c r="B190" t="inlineStr">
         <is>
@@ -4479,14 +4483,14 @@
       </c>
       <c r="D190" t="inlineStr">
         <is>
-          <t>Msc</t>
+          <t>Isl</t>
         </is>
       </c>
       <c r="E190" t="inlineStr"/>
     </row>
     <row r="191">
       <c r="A191" t="n">
-        <v>860054</v>
+        <v>637454</v>
       </c>
       <c r="B191" t="inlineStr">
         <is>
@@ -4495,19 +4499,19 @@
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>Female</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D191" t="inlineStr">
         <is>
-          <t>Msc</t>
+          <t>Isl</t>
         </is>
       </c>
       <c r="E191" t="inlineStr"/>
     </row>
     <row r="192">
       <c r="A192" t="n">
-        <v>597905</v>
+        <v>311140</v>
       </c>
       <c r="B192" t="inlineStr">
         <is>
@@ -4516,23 +4520,19 @@
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>Male</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D192" t="inlineStr">
         <is>
-          <t>Isl</t>
-        </is>
-      </c>
-      <c r="E192" t="inlineStr">
-        <is>
-          <t>Weak in studies</t>
-        </is>
-      </c>
+          <t>Msc</t>
+        </is>
+      </c>
+      <c r="E192" t="inlineStr"/>
     </row>
     <row r="193">
       <c r="A193" t="n">
-        <v>125722</v>
+        <v>194042</v>
       </c>
       <c r="B193" t="inlineStr">
         <is>
@@ -4553,7 +4553,7 @@
     </row>
     <row r="194">
       <c r="A194" t="n">
-        <v>383887</v>
+        <v>781248</v>
       </c>
       <c r="B194" t="inlineStr">
         <is>
@@ -4562,7 +4562,7 @@
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>Male</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D194" t="inlineStr">
@@ -4574,7 +4574,7 @@
     </row>
     <row r="195">
       <c r="A195" t="n">
-        <v>732328</v>
+        <v>453715</v>
       </c>
       <c r="B195" t="inlineStr">
         <is>
@@ -4595,7 +4595,7 @@
     </row>
     <row r="196">
       <c r="A196" t="n">
-        <v>872994</v>
+        <v>149208</v>
       </c>
       <c r="B196" t="inlineStr">
         <is>
@@ -4604,7 +4604,7 @@
       </c>
       <c r="C196" t="inlineStr">
         <is>
-          <t>Female</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D196" t="inlineStr">
@@ -4616,7 +4616,7 @@
     </row>
     <row r="197">
       <c r="A197" t="n">
-        <v>676692</v>
+        <v>672484</v>
       </c>
       <c r="B197" t="inlineStr">
         <is>
@@ -4630,14 +4630,14 @@
       </c>
       <c r="D197" t="inlineStr">
         <is>
-          <t>Msc</t>
+          <t>Isl</t>
         </is>
       </c>
       <c r="E197" t="inlineStr"/>
     </row>
     <row r="198">
       <c r="A198" t="n">
-        <v>442300</v>
+        <v>749136</v>
       </c>
       <c r="B198" t="inlineStr">
         <is>
@@ -4651,14 +4651,14 @@
       </c>
       <c r="D198" t="inlineStr">
         <is>
-          <t>Msc</t>
+          <t>Isl</t>
         </is>
       </c>
       <c r="E198" t="inlineStr"/>
     </row>
     <row r="199">
       <c r="A199" t="n">
-        <v>869162</v>
+        <v>239857</v>
       </c>
       <c r="B199" t="inlineStr">
         <is>
@@ -4667,7 +4667,7 @@
       </c>
       <c r="C199" t="inlineStr">
         <is>
-          <t>Male</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D199" t="inlineStr">
@@ -4679,7 +4679,7 @@
     </row>
     <row r="200">
       <c r="A200" t="n">
-        <v>257343</v>
+        <v>959347</v>
       </c>
       <c r="B200" t="inlineStr">
         <is>
@@ -4688,7 +4688,7 @@
       </c>
       <c r="C200" t="inlineStr">
         <is>
-          <t>Male</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D200" t="inlineStr">
@@ -4700,7 +4700,7 @@
     </row>
     <row r="201">
       <c r="A201" t="n">
-        <v>672651</v>
+        <v>204913</v>
       </c>
       <c r="B201" t="inlineStr">
         <is>
@@ -4709,7 +4709,7 @@
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>Female</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D201" t="inlineStr">
@@ -4721,7 +4721,7 @@
     </row>
     <row r="202">
       <c r="A202" t="n">
-        <v>952198</v>
+        <v>294907</v>
       </c>
       <c r="B202" t="inlineStr">
         <is>
@@ -4742,7 +4742,7 @@
     </row>
     <row r="203">
       <c r="A203" t="n">
-        <v>866290</v>
+        <v>121123</v>
       </c>
       <c r="B203" t="inlineStr">
         <is>
@@ -4751,7 +4751,7 @@
       </c>
       <c r="C203" t="inlineStr">
         <is>
-          <t>Male</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D203" t="inlineStr">
@@ -4763,7 +4763,7 @@
     </row>
     <row r="204">
       <c r="A204" t="n">
-        <v>973268</v>
+        <v>397175</v>
       </c>
       <c r="B204" t="inlineStr">
         <is>
@@ -4772,19 +4772,19 @@
       </c>
       <c r="C204" t="inlineStr">
         <is>
-          <t>Female</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D204" t="inlineStr">
         <is>
-          <t>Isl</t>
+          <t>Msc</t>
         </is>
       </c>
       <c r="E204" t="inlineStr"/>
     </row>
     <row r="205">
       <c r="A205" t="n">
-        <v>707657</v>
+        <v>151643</v>
       </c>
       <c r="B205" t="inlineStr">
         <is>
@@ -4793,7 +4793,7 @@
       </c>
       <c r="C205" t="inlineStr">
         <is>
-          <t>Male</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D205" t="inlineStr">
@@ -4805,7 +4805,7 @@
     </row>
     <row r="206">
       <c r="A206" t="n">
-        <v>222902</v>
+        <v>277160</v>
       </c>
       <c r="B206" t="inlineStr">
         <is>
@@ -4814,544 +4814,19 @@
       </c>
       <c r="C206" t="inlineStr">
         <is>
-          <t>Female</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D206" t="inlineStr">
         <is>
-          <t>Isl</t>
-        </is>
-      </c>
-      <c r="E206" t="inlineStr"/>
-    </row>
-    <row r="207">
-      <c r="A207" t="n">
-        <v>328330</v>
-      </c>
-      <c r="B207" t="inlineStr">
-        <is>
-          <t>Student 206</t>
-        </is>
-      </c>
-      <c r="C207" t="inlineStr">
-        <is>
-          <t>Female</t>
-        </is>
-      </c>
-      <c r="D207" t="inlineStr">
-        <is>
-          <t>Msc</t>
-        </is>
-      </c>
-      <c r="E207" t="inlineStr"/>
-    </row>
-    <row r="208">
-      <c r="A208" t="n">
-        <v>299729</v>
-      </c>
-      <c r="B208" t="inlineStr">
-        <is>
-          <t>Student 207</t>
-        </is>
-      </c>
-      <c r="C208" t="inlineStr">
-        <is>
-          <t>Female</t>
-        </is>
-      </c>
-      <c r="D208" t="inlineStr">
-        <is>
-          <t>Msc</t>
-        </is>
-      </c>
-      <c r="E208" t="inlineStr"/>
-    </row>
-    <row r="209">
-      <c r="A209" t="n">
-        <v>102486</v>
-      </c>
-      <c r="B209" t="inlineStr">
-        <is>
-          <t>Student 208</t>
-        </is>
-      </c>
-      <c r="C209" t="inlineStr">
-        <is>
-          <t>Female</t>
-        </is>
-      </c>
-      <c r="D209" t="inlineStr">
-        <is>
-          <t>Msc</t>
-        </is>
-      </c>
-      <c r="E209" t="inlineStr"/>
-    </row>
-    <row r="210">
-      <c r="A210" t="n">
-        <v>397077</v>
-      </c>
-      <c r="B210" t="inlineStr">
-        <is>
-          <t>Student 209</t>
-        </is>
-      </c>
-      <c r="C210" t="inlineStr">
-        <is>
-          <t>Male</t>
-        </is>
-      </c>
-      <c r="D210" t="inlineStr">
-        <is>
-          <t>Isl</t>
-        </is>
-      </c>
-      <c r="E210" t="inlineStr"/>
-    </row>
-    <row r="211">
-      <c r="A211" t="n">
-        <v>762964</v>
-      </c>
-      <c r="B211" t="inlineStr">
-        <is>
-          <t>Student 210</t>
-        </is>
-      </c>
-      <c r="C211" t="inlineStr">
-        <is>
-          <t>Male</t>
-        </is>
-      </c>
-      <c r="D211" t="inlineStr">
-        <is>
-          <t>Msc</t>
-        </is>
-      </c>
-      <c r="E211" t="inlineStr"/>
-    </row>
-    <row r="212">
-      <c r="A212" t="n">
-        <v>635051</v>
-      </c>
-      <c r="B212" t="inlineStr">
-        <is>
-          <t>Student 211</t>
-        </is>
-      </c>
-      <c r="C212" t="inlineStr">
-        <is>
-          <t>Female</t>
-        </is>
-      </c>
-      <c r="D212" t="inlineStr">
-        <is>
-          <t>Msc</t>
-        </is>
-      </c>
-      <c r="E212" t="inlineStr"/>
-    </row>
-    <row r="213">
-      <c r="A213" t="n">
-        <v>736173</v>
-      </c>
-      <c r="B213" t="inlineStr">
-        <is>
-          <t>Student 212</t>
-        </is>
-      </c>
-      <c r="C213" t="inlineStr">
-        <is>
-          <t>Female</t>
-        </is>
-      </c>
-      <c r="D213" t="inlineStr">
-        <is>
-          <t>Isl</t>
-        </is>
-      </c>
-      <c r="E213" t="inlineStr"/>
-    </row>
-    <row r="214">
-      <c r="A214" t="n">
-        <v>799937</v>
-      </c>
-      <c r="B214" t="inlineStr">
-        <is>
-          <t>Student 213</t>
-        </is>
-      </c>
-      <c r="C214" t="inlineStr">
-        <is>
-          <t>Female</t>
-        </is>
-      </c>
-      <c r="D214" t="inlineStr">
-        <is>
-          <t>Msc</t>
-        </is>
-      </c>
-      <c r="E214" t="inlineStr"/>
-    </row>
-    <row r="215">
-      <c r="A215" t="n">
-        <v>783822</v>
-      </c>
-      <c r="B215" t="inlineStr">
-        <is>
-          <t>Student 214</t>
-        </is>
-      </c>
-      <c r="C215" t="inlineStr">
-        <is>
-          <t>Female</t>
-        </is>
-      </c>
-      <c r="D215" t="inlineStr">
-        <is>
-          <t>Isl</t>
-        </is>
-      </c>
-      <c r="E215" t="inlineStr"/>
-    </row>
-    <row r="216">
-      <c r="A216" t="n">
-        <v>212203</v>
-      </c>
-      <c r="B216" t="inlineStr">
-        <is>
-          <t>Student 215</t>
-        </is>
-      </c>
-      <c r="C216" t="inlineStr">
-        <is>
-          <t>Female</t>
-        </is>
-      </c>
-      <c r="D216" t="inlineStr">
-        <is>
-          <t>Msc</t>
-        </is>
-      </c>
-      <c r="E216" t="inlineStr"/>
-    </row>
-    <row r="217">
-      <c r="A217" t="n">
-        <v>886022</v>
-      </c>
-      <c r="B217" t="inlineStr">
-        <is>
-          <t>Student 216</t>
-        </is>
-      </c>
-      <c r="C217" t="inlineStr">
-        <is>
-          <t>Male</t>
-        </is>
-      </c>
-      <c r="D217" t="inlineStr">
-        <is>
-          <t>Isl</t>
-        </is>
-      </c>
-      <c r="E217" t="inlineStr"/>
-    </row>
-    <row r="218">
-      <c r="A218" t="n">
-        <v>865953</v>
-      </c>
-      <c r="B218" t="inlineStr">
-        <is>
-          <t>Student 217</t>
-        </is>
-      </c>
-      <c r="C218" t="inlineStr">
-        <is>
-          <t>Female</t>
-        </is>
-      </c>
-      <c r="D218" t="inlineStr">
-        <is>
-          <t>Msc</t>
-        </is>
-      </c>
-      <c r="E218" t="inlineStr"/>
-    </row>
-    <row r="219">
-      <c r="A219" t="n">
-        <v>541391</v>
-      </c>
-      <c r="B219" t="inlineStr">
-        <is>
-          <t>Student 218</t>
-        </is>
-      </c>
-      <c r="C219" t="inlineStr">
-        <is>
-          <t>Male</t>
-        </is>
-      </c>
-      <c r="D219" t="inlineStr">
-        <is>
-          <t>Msc</t>
-        </is>
-      </c>
-      <c r="E219" t="inlineStr"/>
-    </row>
-    <row r="220">
-      <c r="A220" t="n">
-        <v>993257</v>
-      </c>
-      <c r="B220" t="inlineStr">
-        <is>
-          <t>Student 219</t>
-        </is>
-      </c>
-      <c r="C220" t="inlineStr">
-        <is>
-          <t>Male</t>
-        </is>
-      </c>
-      <c r="D220" t="inlineStr">
-        <is>
-          <t>Msc</t>
-        </is>
-      </c>
-      <c r="E220" t="inlineStr"/>
-    </row>
-    <row r="221">
-      <c r="A221" t="n">
-        <v>515105</v>
-      </c>
-      <c r="B221" t="inlineStr">
-        <is>
-          <t>Student 220</t>
-        </is>
-      </c>
-      <c r="C221" t="inlineStr">
-        <is>
-          <t>Male</t>
-        </is>
-      </c>
-      <c r="D221" t="inlineStr">
-        <is>
-          <t>Msc</t>
-        </is>
-      </c>
-      <c r="E221" t="inlineStr"/>
-    </row>
-    <row r="222">
-      <c r="A222" t="n">
-        <v>709207</v>
-      </c>
-      <c r="B222" t="inlineStr">
-        <is>
-          <t>Student 221</t>
-        </is>
-      </c>
-      <c r="C222" t="inlineStr">
-        <is>
-          <t>Male</t>
-        </is>
-      </c>
-      <c r="D222" t="inlineStr">
-        <is>
-          <t>Isl</t>
-        </is>
-      </c>
-      <c r="E222" t="inlineStr"/>
-    </row>
-    <row r="223">
-      <c r="A223" t="n">
-        <v>811651</v>
-      </c>
-      <c r="B223" t="inlineStr">
-        <is>
-          <t>Student 222</t>
-        </is>
-      </c>
-      <c r="C223" t="inlineStr">
-        <is>
-          <t>Female</t>
-        </is>
-      </c>
-      <c r="D223" t="inlineStr">
-        <is>
-          <t>Isl</t>
-        </is>
-      </c>
-      <c r="E223" t="inlineStr"/>
-    </row>
-    <row r="224">
-      <c r="A224" t="n">
-        <v>899577</v>
-      </c>
-      <c r="B224" t="inlineStr">
-        <is>
-          <t>Student 223</t>
-        </is>
-      </c>
-      <c r="C224" t="inlineStr">
-        <is>
-          <t>Male</t>
-        </is>
-      </c>
-      <c r="D224" t="inlineStr">
-        <is>
-          <t>Msc</t>
-        </is>
-      </c>
-      <c r="E224" t="inlineStr">
-        <is>
-          <t>Naughty</t>
-        </is>
-      </c>
-    </row>
-    <row r="225">
-      <c r="A225" t="n">
-        <v>519569</v>
-      </c>
-      <c r="B225" t="inlineStr">
-        <is>
-          <t>Student 224</t>
-        </is>
-      </c>
-      <c r="C225" t="inlineStr">
-        <is>
-          <t>Female</t>
-        </is>
-      </c>
-      <c r="D225" t="inlineStr">
-        <is>
-          <t>Msc</t>
-        </is>
-      </c>
-      <c r="E225" t="inlineStr"/>
-    </row>
-    <row r="226">
-      <c r="A226" t="n">
-        <v>570099</v>
-      </c>
-      <c r="B226" t="inlineStr">
-        <is>
-          <t>Student 225</t>
-        </is>
-      </c>
-      <c r="C226" t="inlineStr">
-        <is>
-          <t>Female</t>
-        </is>
-      </c>
-      <c r="D226" t="inlineStr">
-        <is>
-          <t>Msc</t>
-        </is>
-      </c>
-      <c r="E226" t="inlineStr"/>
-    </row>
-    <row r="227">
-      <c r="A227" t="n">
-        <v>422371</v>
-      </c>
-      <c r="B227" t="inlineStr">
-        <is>
-          <t>Student 226</t>
-        </is>
-      </c>
-      <c r="C227" t="inlineStr">
-        <is>
-          <t>Male</t>
-        </is>
-      </c>
-      <c r="D227" t="inlineStr">
-        <is>
-          <t>Msc</t>
-        </is>
-      </c>
-      <c r="E227" t="inlineStr"/>
-    </row>
-    <row r="228">
-      <c r="A228" t="n">
-        <v>886375</v>
-      </c>
-      <c r="B228" t="inlineStr">
-        <is>
-          <t>Student 227</t>
-        </is>
-      </c>
-      <c r="C228" t="inlineStr">
-        <is>
-          <t>Female</t>
-        </is>
-      </c>
-      <c r="D228" t="inlineStr">
-        <is>
-          <t>Msc</t>
-        </is>
-      </c>
-      <c r="E228" t="inlineStr"/>
-    </row>
-    <row r="229">
-      <c r="A229" t="n">
-        <v>593135</v>
-      </c>
-      <c r="B229" t="inlineStr">
-        <is>
-          <t>Student 228</t>
-        </is>
-      </c>
-      <c r="C229" t="inlineStr">
-        <is>
-          <t>Male</t>
-        </is>
-      </c>
-      <c r="D229" t="inlineStr">
-        <is>
-          <t>Msc</t>
-        </is>
-      </c>
-      <c r="E229" t="inlineStr"/>
-    </row>
-    <row r="230">
-      <c r="A230" t="n">
-        <v>767757</v>
-      </c>
-      <c r="B230" t="inlineStr">
-        <is>
-          <t>Student 229</t>
-        </is>
-      </c>
-      <c r="C230" t="inlineStr">
-        <is>
-          <t>Male</t>
-        </is>
-      </c>
-      <c r="D230" t="inlineStr">
-        <is>
-          <t>Msc</t>
-        </is>
-      </c>
-      <c r="E230" t="inlineStr"/>
-    </row>
-    <row r="231">
-      <c r="A231" t="n">
-        <v>952080</v>
-      </c>
-      <c r="B231" t="inlineStr">
-        <is>
-          <t>Student 230</t>
-        </is>
-      </c>
-      <c r="C231" t="inlineStr">
-        <is>
-          <t>Male</t>
-        </is>
-      </c>
-      <c r="D231" t="inlineStr">
-        <is>
-          <t>Isl</t>
-        </is>
-      </c>
-      <c r="E231" t="inlineStr"/>
+          <t>Msc</t>
+        </is>
+      </c>
+      <c r="E206" t="inlineStr">
+        <is>
+          <t>Weak in studies</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>